<commit_message>
Cambiamos la definicion de la tabla para que todas fechas sean timestamps, ya lo manejamos asi en el código. Agregamos más fechas en los historicos de velas.
</commit_message>
<xml_diff>
--- a/Historico de Fibras.xlsx
+++ b/Historico de Fibras.xlsx
@@ -8,21 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\M R\Documents\Python\BDHistorico\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F57A7F54-1B2F-4C16-BFA3-039296A26224}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CEA67E4-FA16-4084-A307-3A44AACBBFDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="15600" windowHeight="19440" tabRatio="705" activeTab="1" xr2:uid="{61FC1FF2-927D-4FA9-8C22-EC769C0CC026}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="15600" windowHeight="19440" tabRatio="705" activeTab="2" xr2:uid="{61FC1FF2-927D-4FA9-8C22-EC769C0CC026}"/>
   </bookViews>
   <sheets>
     <sheet name="Fechas de distribucion" sheetId="1" r:id="rId1"/>
     <sheet name="FCFE18" sheetId="9" r:id="rId2"/>
-    <sheet name="FIHO12" sheetId="7" r:id="rId3"/>
-    <sheet name="FIBRAPL14" sheetId="2" r:id="rId4"/>
-    <sheet name="FUNO11" sheetId="3" r:id="rId5"/>
-    <sheet name="FMTY14" sheetId="4" r:id="rId6"/>
-    <sheet name="FNOVA17" sheetId="10" r:id="rId7"/>
-    <sheet name="FIBRAMQ12" sheetId="5" r:id="rId8"/>
-    <sheet name="FHIPO14" sheetId="6" r:id="rId9"/>
-    <sheet name="DANHOS13" sheetId="8" r:id="rId10"/>
+    <sheet name="FIBRATC14" sheetId="11" r:id="rId3"/>
+    <sheet name="FIHO12" sheetId="7" r:id="rId4"/>
+    <sheet name="FIBRAPL14" sheetId="2" r:id="rId5"/>
+    <sheet name="FUNO11" sheetId="3" r:id="rId6"/>
+    <sheet name="FMTY14" sheetId="4" r:id="rId7"/>
+    <sheet name="FNOVA17" sheetId="10" r:id="rId8"/>
+    <sheet name="FIBRAMQ12" sheetId="5" r:id="rId9"/>
+    <sheet name="FHIPO14" sheetId="6" r:id="rId10"/>
+    <sheet name="DANHOS13" sheetId="8" r:id="rId11"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="579" uniqueCount="87">
   <si>
     <t>ENERO</t>
   </si>
@@ -292,6 +293,9 @@
   </si>
   <si>
     <t>FNOVA17</t>
+  </si>
+  <si>
+    <t>FIBRATC14</t>
   </si>
 </sst>
 </file>
@@ -1386,6 +1390,363 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{200EB5CF-E323-4820-B096-9F8315944A3A}">
+  <dimension ref="A1:E20"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D2" t="s">
+        <v>79</v>
+      </c>
+      <c r="E2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="3">
+        <v>45791</v>
+      </c>
+      <c r="B3">
+        <v>0.32</v>
+      </c>
+      <c r="C3" t="s">
+        <v>74</v>
+      </c>
+      <c r="D3" s="3">
+        <v>45792</v>
+      </c>
+      <c r="E3">
+        <v>9.0499999999999997E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="3">
+        <v>45728</v>
+      </c>
+      <c r="B4">
+        <v>0.12</v>
+      </c>
+      <c r="C4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D4" s="3">
+        <v>45729</v>
+      </c>
+      <c r="E4">
+        <v>3.7400000000000003E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="3">
+        <v>45616</v>
+      </c>
+      <c r="B5">
+        <v>0.4</v>
+      </c>
+      <c r="C5" t="s">
+        <v>74</v>
+      </c>
+      <c r="D5" s="3">
+        <v>45617</v>
+      </c>
+      <c r="E5">
+        <v>9.6199999999999994E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="3">
+        <v>45518</v>
+      </c>
+      <c r="B6">
+        <v>0.33</v>
+      </c>
+      <c r="C6" t="s">
+        <v>74</v>
+      </c>
+      <c r="D6" s="3">
+        <v>45519</v>
+      </c>
+      <c r="E6">
+        <v>7.9600000000000004E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="3">
+        <v>45426</v>
+      </c>
+      <c r="B7">
+        <v>0.36</v>
+      </c>
+      <c r="C7" t="s">
+        <v>74</v>
+      </c>
+      <c r="D7" s="3">
+        <v>45428</v>
+      </c>
+      <c r="E7">
+        <v>8.6099999999999996E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="3">
+        <v>45357</v>
+      </c>
+      <c r="B8">
+        <v>0.5</v>
+      </c>
+      <c r="C8" t="s">
+        <v>74</v>
+      </c>
+      <c r="D8" s="3">
+        <v>45359</v>
+      </c>
+      <c r="E8">
+        <v>0.1246</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="3">
+        <v>45244</v>
+      </c>
+      <c r="B9">
+        <v>0.68</v>
+      </c>
+      <c r="C9" t="s">
+        <v>74</v>
+      </c>
+      <c r="D9" s="3">
+        <v>45246</v>
+      </c>
+      <c r="E9">
+        <v>0.15920000000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="3">
+        <v>45153</v>
+      </c>
+      <c r="B10">
+        <v>0.48</v>
+      </c>
+      <c r="C10" t="s">
+        <v>74</v>
+      </c>
+      <c r="D10" s="3">
+        <v>45155</v>
+      </c>
+      <c r="E10">
+        <v>0.1106</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="3">
+        <v>45062</v>
+      </c>
+      <c r="B11">
+        <v>0.26</v>
+      </c>
+      <c r="C11" t="s">
+        <v>74</v>
+      </c>
+      <c r="D11" s="3">
+        <v>45064</v>
+      </c>
+      <c r="E11">
+        <v>6.0699999999999997E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="3">
+        <v>44999</v>
+      </c>
+      <c r="B12">
+        <v>0.62</v>
+      </c>
+      <c r="C12" t="s">
+        <v>74</v>
+      </c>
+      <c r="D12" s="3">
+        <v>45001</v>
+      </c>
+      <c r="E12">
+        <v>0.14480000000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="3">
+        <v>44880</v>
+      </c>
+      <c r="B13">
+        <v>0.47</v>
+      </c>
+      <c r="C13" t="s">
+        <v>74</v>
+      </c>
+      <c r="D13" s="3">
+        <v>44882</v>
+      </c>
+      <c r="E13">
+        <v>0.1014</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="3">
+        <v>44789</v>
+      </c>
+      <c r="B14">
+        <v>0.71</v>
+      </c>
+      <c r="C14" t="s">
+        <v>74</v>
+      </c>
+      <c r="D14" s="3">
+        <v>44791</v>
+      </c>
+      <c r="E14">
+        <v>0.1512</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="3">
+        <v>44698</v>
+      </c>
+      <c r="B15">
+        <v>0.47</v>
+      </c>
+      <c r="C15" t="s">
+        <v>74</v>
+      </c>
+      <c r="D15" s="3">
+        <v>44700</v>
+      </c>
+      <c r="E15">
+        <v>9.69E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="3">
+        <v>44271</v>
+      </c>
+      <c r="B16">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="C16" t="s">
+        <v>74</v>
+      </c>
+      <c r="D16" s="3">
+        <v>44273</v>
+      </c>
+      <c r="E16">
+        <v>5.6500000000000002E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="3">
+        <v>44152</v>
+      </c>
+      <c r="B17">
+        <v>0.34</v>
+      </c>
+      <c r="C17" t="s">
+        <v>74</v>
+      </c>
+      <c r="D17" s="3">
+        <v>44154</v>
+      </c>
+      <c r="E17">
+        <v>7.5300000000000006E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="3">
+        <v>44061</v>
+      </c>
+      <c r="B18">
+        <v>0.39</v>
+      </c>
+      <c r="C18" t="s">
+        <v>74</v>
+      </c>
+      <c r="D18" s="3">
+        <v>44063</v>
+      </c>
+      <c r="E18">
+        <v>8.7800000000000003E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="3">
+        <v>43970</v>
+      </c>
+      <c r="B19">
+        <v>0.46</v>
+      </c>
+      <c r="C19" t="s">
+        <v>74</v>
+      </c>
+      <c r="D19" s="3">
+        <v>43972</v>
+      </c>
+      <c r="E19">
+        <v>0.11509999999999999</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="3">
+        <v>43909</v>
+      </c>
+      <c r="B20">
+        <v>0.11</v>
+      </c>
+      <c r="C20" t="s">
+        <v>74</v>
+      </c>
+      <c r="D20" s="3">
+        <v>43913</v>
+      </c>
+      <c r="E20">
+        <v>2.53E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AC2906F-15DF-4E52-ACB6-A604BEFC7F04}">
   <dimension ref="A1:E16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1980,6 +2341,1876 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AB83DE9-234F-4FC9-8EC0-C932B00F0E83}">
+  <dimension ref="A1:E109"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C1" t="s">
+        <v>86</v>
+      </c>
+      <c r="D1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D2" t="s">
+        <v>79</v>
+      </c>
+      <c r="E2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="3">
+        <v>45884</v>
+      </c>
+      <c r="B3">
+        <v>0.06</v>
+      </c>
+      <c r="C3" t="s">
+        <v>76</v>
+      </c>
+      <c r="D3" s="3">
+        <v>45887</v>
+      </c>
+      <c r="E3">
+        <v>6.6299999999999998E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="3">
+        <v>45880</v>
+      </c>
+      <c r="B4">
+        <v>0.16</v>
+      </c>
+      <c r="C4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D4" s="3">
+        <v>45881</v>
+      </c>
+      <c r="E4">
+        <v>6.4699999999999994E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="3">
+        <v>45870</v>
+      </c>
+      <c r="B5">
+        <v>0.01</v>
+      </c>
+      <c r="C5" t="s">
+        <v>75</v>
+      </c>
+      <c r="D5" s="3">
+        <v>45873</v>
+      </c>
+      <c r="E5">
+        <v>5.4899999999999997E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="3">
+        <v>45868</v>
+      </c>
+      <c r="B6">
+        <v>0.04</v>
+      </c>
+      <c r="C6" t="s">
+        <v>75</v>
+      </c>
+      <c r="D6" s="3">
+        <v>45869</v>
+      </c>
+      <c r="E6">
+        <v>5.6099999999999997E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="3">
+        <v>45841</v>
+      </c>
+      <c r="B7">
+        <v>0.04</v>
+      </c>
+      <c r="C7" t="s">
+        <v>75</v>
+      </c>
+      <c r="D7" s="3">
+        <v>45842</v>
+      </c>
+      <c r="E7">
+        <v>6.8000000000000005E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="3">
+        <v>45840</v>
+      </c>
+      <c r="B8">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="C8" t="s">
+        <v>76</v>
+      </c>
+      <c r="D8" s="3">
+        <v>45841</v>
+      </c>
+      <c r="E8">
+        <v>6.5100000000000005E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="3">
+        <v>45814</v>
+      </c>
+      <c r="B9">
+        <v>0.04</v>
+      </c>
+      <c r="C9" t="s">
+        <v>75</v>
+      </c>
+      <c r="D9" s="3">
+        <v>45817</v>
+      </c>
+      <c r="E9">
+        <v>6.0699999999999997E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="3">
+        <v>45789</v>
+      </c>
+      <c r="B10">
+        <v>0.13</v>
+      </c>
+      <c r="C10" t="s">
+        <v>75</v>
+      </c>
+      <c r="D10" s="3">
+        <v>45790</v>
+      </c>
+      <c r="E10">
+        <v>6.3200000000000006E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="3">
+        <v>45785</v>
+      </c>
+      <c r="B11">
+        <v>0.15</v>
+      </c>
+      <c r="C11" t="s">
+        <v>75</v>
+      </c>
+      <c r="D11" s="3">
+        <v>45786</v>
+      </c>
+      <c r="E11">
+        <v>5.7099999999999998E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="3">
+        <v>45728</v>
+      </c>
+      <c r="B12">
+        <v>0.15</v>
+      </c>
+      <c r="C12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D12" s="3">
+        <v>45729</v>
+      </c>
+      <c r="E12">
+        <v>6.6199999999999995E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="3">
+        <v>45722</v>
+      </c>
+      <c r="B13">
+        <v>0.03</v>
+      </c>
+      <c r="C13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D13" s="3">
+        <v>45723</v>
+      </c>
+      <c r="E13">
+        <v>5.8700000000000002E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="3">
+        <v>45701</v>
+      </c>
+      <c r="B14">
+        <v>0.21</v>
+      </c>
+      <c r="C14" t="s">
+        <v>75</v>
+      </c>
+      <c r="D14" s="3">
+        <v>45702</v>
+      </c>
+      <c r="E14">
+        <v>7.1900000000000006E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="3">
+        <v>45693</v>
+      </c>
+      <c r="B15">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="C15" t="s">
+        <v>75</v>
+      </c>
+      <c r="D15" s="3">
+        <v>45694</v>
+      </c>
+      <c r="E15">
+        <v>7.7700000000000005E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="3">
+        <v>45643</v>
+      </c>
+      <c r="B16">
+        <v>0.01</v>
+      </c>
+      <c r="C16" t="s">
+        <v>75</v>
+      </c>
+      <c r="D16" s="3">
+        <v>45644</v>
+      </c>
+      <c r="E16">
+        <v>9.3200000000000005E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="3">
+        <v>45610</v>
+      </c>
+      <c r="B17">
+        <v>0.05</v>
+      </c>
+      <c r="C17" t="s">
+        <v>75</v>
+      </c>
+      <c r="D17" s="3">
+        <v>45611</v>
+      </c>
+      <c r="E17">
+        <v>9.0300000000000005E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="3">
+        <v>45604</v>
+      </c>
+      <c r="B18">
+        <v>0.13</v>
+      </c>
+      <c r="C18" t="s">
+        <v>76</v>
+      </c>
+      <c r="D18" s="3">
+        <v>45607</v>
+      </c>
+      <c r="E18">
+        <v>8.6400000000000005E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="3">
+        <v>45596</v>
+      </c>
+      <c r="B19">
+        <v>0.06</v>
+      </c>
+      <c r="C19" t="s">
+        <v>75</v>
+      </c>
+      <c r="D19" s="3">
+        <v>45597</v>
+      </c>
+      <c r="E19">
+        <v>8.09E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="3">
+        <v>45572</v>
+      </c>
+      <c r="B20">
+        <v>0.06</v>
+      </c>
+      <c r="C20" t="s">
+        <v>75</v>
+      </c>
+      <c r="D20" s="3">
+        <v>45573</v>
+      </c>
+      <c r="E20">
+        <v>7.6700000000000004E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="3">
+        <v>45547</v>
+      </c>
+      <c r="B21">
+        <v>0.01</v>
+      </c>
+      <c r="C21" t="s">
+        <v>75</v>
+      </c>
+      <c r="D21" s="3">
+        <v>45548</v>
+      </c>
+      <c r="E21">
+        <v>7.6499999999999999E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="3">
+        <v>45523</v>
+      </c>
+      <c r="B22">
+        <v>0.06</v>
+      </c>
+      <c r="C22" t="s">
+        <v>76</v>
+      </c>
+      <c r="D22" s="3">
+        <v>45524</v>
+      </c>
+      <c r="E22">
+        <v>7.2099999999999997E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="3">
+        <v>45518</v>
+      </c>
+      <c r="B23">
+        <v>0.05</v>
+      </c>
+      <c r="C23" t="s">
+        <v>75</v>
+      </c>
+      <c r="D23" s="3">
+        <v>45519</v>
+      </c>
+      <c r="E23">
+        <v>8.5599999999999996E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="3">
+        <v>45512</v>
+      </c>
+      <c r="B24">
+        <v>0.17</v>
+      </c>
+      <c r="C24" t="s">
+        <v>75</v>
+      </c>
+      <c r="D24" s="3">
+        <v>45513</v>
+      </c>
+      <c r="E24">
+        <v>8.5000000000000006E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="3">
+        <v>45471</v>
+      </c>
+      <c r="B25">
+        <v>0.01</v>
+      </c>
+      <c r="C25" t="s">
+        <v>75</v>
+      </c>
+      <c r="D25" s="3">
+        <v>45474</v>
+      </c>
+      <c r="E25">
+        <v>9.0300000000000005E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="3">
+        <v>45457</v>
+      </c>
+      <c r="B26">
+        <v>0.05</v>
+      </c>
+      <c r="C26" t="s">
+        <v>76</v>
+      </c>
+      <c r="D26" s="3">
+        <v>45460</v>
+      </c>
+      <c r="E26">
+        <v>9.3200000000000005E-2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="3">
+        <v>45421</v>
+      </c>
+      <c r="B27">
+        <v>0.06</v>
+      </c>
+      <c r="C27" t="s">
+        <v>75</v>
+      </c>
+      <c r="D27" s="3">
+        <v>45426</v>
+      </c>
+      <c r="E27">
+        <v>8.77E-2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="3">
+        <v>45419</v>
+      </c>
+      <c r="B28">
+        <v>0.13</v>
+      </c>
+      <c r="C28" t="s">
+        <v>76</v>
+      </c>
+      <c r="D28" s="3">
+        <v>45421</v>
+      </c>
+      <c r="E28">
+        <v>8.4099999999999994E-2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" s="3">
+        <v>45414</v>
+      </c>
+      <c r="B29">
+        <v>0.04</v>
+      </c>
+      <c r="C29" t="s">
+        <v>76</v>
+      </c>
+      <c r="D29" s="3">
+        <v>45418</v>
+      </c>
+      <c r="E29">
+        <v>7.3400000000000007E-2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" s="3">
+        <v>45408</v>
+      </c>
+      <c r="B30">
+        <v>0</v>
+      </c>
+      <c r="C30" t="s">
+        <v>75</v>
+      </c>
+      <c r="D30" s="3">
+        <v>45412</v>
+      </c>
+      <c r="E30">
+        <v>7.51E-2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="3">
+        <v>45364</v>
+      </c>
+      <c r="B31">
+        <v>0.02</v>
+      </c>
+      <c r="C31" t="s">
+        <v>76</v>
+      </c>
+      <c r="D31" s="3">
+        <v>45366</v>
+      </c>
+      <c r="E31">
+        <v>7.9899999999999999E-2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="3">
+        <v>45363</v>
+      </c>
+      <c r="B32">
+        <v>0.23</v>
+      </c>
+      <c r="C32" t="s">
+        <v>76</v>
+      </c>
+      <c r="D32" s="3">
+        <v>45365</v>
+      </c>
+      <c r="E32">
+        <v>7.8399999999999997E-2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="3">
+        <v>45357</v>
+      </c>
+      <c r="B33">
+        <v>0.05</v>
+      </c>
+      <c r="C33" t="s">
+        <v>76</v>
+      </c>
+      <c r="D33" s="3">
+        <v>45359</v>
+      </c>
+      <c r="E33">
+        <v>6.8699999999999997E-2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="3">
+        <v>45355</v>
+      </c>
+      <c r="B34">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="C34" t="s">
+        <v>76</v>
+      </c>
+      <c r="D34" s="3">
+        <v>45357</v>
+      </c>
+      <c r="E34">
+        <v>6.5600000000000006E-2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="3">
+        <v>45352</v>
+      </c>
+      <c r="B35">
+        <v>0.04</v>
+      </c>
+      <c r="C35" t="s">
+        <v>76</v>
+      </c>
+      <c r="D35" s="3">
+        <v>45356</v>
+      </c>
+      <c r="E35">
+        <v>5.4600000000000003E-2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" s="3">
+        <v>45341</v>
+      </c>
+      <c r="B36">
+        <v>0.1</v>
+      </c>
+      <c r="C36" t="s">
+        <v>76</v>
+      </c>
+      <c r="D36" s="3">
+        <v>45343</v>
+      </c>
+      <c r="E36">
+        <v>5.33E-2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" s="3">
+        <v>45329</v>
+      </c>
+      <c r="B37">
+        <v>0.12</v>
+      </c>
+      <c r="C37" t="s">
+        <v>76</v>
+      </c>
+      <c r="D37" s="3">
+        <v>45331</v>
+      </c>
+      <c r="E37">
+        <v>5.5E-2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" s="3">
+        <v>45323</v>
+      </c>
+      <c r="B38">
+        <v>0.04</v>
+      </c>
+      <c r="C38" t="s">
+        <v>76</v>
+      </c>
+      <c r="D38" s="3">
+        <v>45328</v>
+      </c>
+      <c r="E38">
+        <v>5.0700000000000002E-2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" s="3">
+        <v>45320</v>
+      </c>
+      <c r="B39">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="C39" t="s">
+        <v>76</v>
+      </c>
+      <c r="D39" s="3">
+        <v>45322</v>
+      </c>
+      <c r="E39">
+        <v>4.8399999999999999E-2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" s="3">
+        <v>45280</v>
+      </c>
+      <c r="B40">
+        <v>0.01</v>
+      </c>
+      <c r="C40" t="s">
+        <v>76</v>
+      </c>
+      <c r="D40" s="3">
+        <v>45282</v>
+      </c>
+      <c r="E40">
+        <v>4.4900000000000002E-2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="3">
+        <v>45244</v>
+      </c>
+      <c r="B41">
+        <v>0.05</v>
+      </c>
+      <c r="C41" t="s">
+        <v>75</v>
+      </c>
+      <c r="D41" s="3">
+        <v>45246</v>
+      </c>
+      <c r="E41">
+        <v>4.87E-2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" s="3">
+        <v>45237</v>
+      </c>
+      <c r="B42">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="C42" t="s">
+        <v>75</v>
+      </c>
+      <c r="D42" s="3">
+        <v>45239</v>
+      </c>
+      <c r="E42">
+        <v>4.6300000000000001E-2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" s="3">
+        <v>45236</v>
+      </c>
+      <c r="B43">
+        <v>0.03</v>
+      </c>
+      <c r="C43" t="s">
+        <v>76</v>
+      </c>
+      <c r="D43" s="3">
+        <v>45238</v>
+      </c>
+      <c r="E43">
+        <v>5.2999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" s="3">
+        <v>45230</v>
+      </c>
+      <c r="B44">
+        <v>0.05</v>
+      </c>
+      <c r="C44" t="s">
+        <v>76</v>
+      </c>
+      <c r="D44" s="3">
+        <v>45233</v>
+      </c>
+      <c r="E44">
+        <v>5.5599999999999997E-2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" s="3">
+        <v>45196</v>
+      </c>
+      <c r="B45">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="C45" t="s">
+        <v>75</v>
+      </c>
+      <c r="D45" s="3">
+        <v>45198</v>
+      </c>
+      <c r="E45">
+        <v>6.6900000000000001E-2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" s="3">
+        <v>45147</v>
+      </c>
+      <c r="B46">
+        <v>0.06</v>
+      </c>
+      <c r="C46" t="s">
+        <v>76</v>
+      </c>
+      <c r="D46" s="3">
+        <v>45149</v>
+      </c>
+      <c r="E46">
+        <v>6.7000000000000004E-2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" s="3">
+        <v>45145</v>
+      </c>
+      <c r="B47">
+        <v>0.16</v>
+      </c>
+      <c r="C47" t="s">
+        <v>76</v>
+      </c>
+      <c r="D47" s="3">
+        <v>45147</v>
+      </c>
+      <c r="E47">
+        <v>6.3500000000000001E-2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" s="3">
+        <v>45134</v>
+      </c>
+      <c r="B48">
+        <v>0.05</v>
+      </c>
+      <c r="C48" t="s">
+        <v>76</v>
+      </c>
+      <c r="D48" s="3">
+        <v>45138</v>
+      </c>
+      <c r="E48">
+        <v>5.5300000000000002E-2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" s="3">
+        <v>45093</v>
+      </c>
+      <c r="B49">
+        <v>0.05</v>
+      </c>
+      <c r="C49" t="s">
+        <v>76</v>
+      </c>
+      <c r="D49" s="3">
+        <v>45097</v>
+      </c>
+      <c r="E49">
+        <v>6.7000000000000004E-2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" s="3">
+        <v>45058</v>
+      </c>
+      <c r="B50">
+        <v>0.05</v>
+      </c>
+      <c r="C50" t="s">
+        <v>76</v>
+      </c>
+      <c r="D50" s="3">
+        <v>45062</v>
+      </c>
+      <c r="E50">
+        <v>6.8400000000000002E-2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" s="3">
+        <v>45055</v>
+      </c>
+      <c r="B51">
+        <v>0.01</v>
+      </c>
+      <c r="C51" t="s">
+        <v>76</v>
+      </c>
+      <c r="D51" s="3">
+        <v>45057</v>
+      </c>
+      <c r="E51">
+        <v>6.54E-2</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" s="3">
+        <v>45054</v>
+      </c>
+      <c r="B52">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="C52" t="s">
+        <v>76</v>
+      </c>
+      <c r="D52" s="3">
+        <v>45056</v>
+      </c>
+      <c r="E52">
+        <v>6.5100000000000005E-2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" s="3">
+        <v>45021</v>
+      </c>
+      <c r="B53">
+        <v>0.01</v>
+      </c>
+      <c r="C53" t="s">
+        <v>76</v>
+      </c>
+      <c r="D53" s="3">
+        <v>45027</v>
+      </c>
+      <c r="E53">
+        <v>7.0699999999999999E-2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" s="3">
+        <v>44998</v>
+      </c>
+      <c r="B54">
+        <v>0.03</v>
+      </c>
+      <c r="C54" t="s">
+        <v>76</v>
+      </c>
+      <c r="D54" s="3">
+        <v>45000</v>
+      </c>
+      <c r="E54">
+        <v>6.9400000000000003E-2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55" s="3">
+        <v>44991</v>
+      </c>
+      <c r="B55">
+        <v>0.06</v>
+      </c>
+      <c r="C55" t="s">
+        <v>75</v>
+      </c>
+      <c r="D55" s="3">
+        <v>44993</v>
+      </c>
+      <c r="E55">
+        <v>6.6000000000000003E-2</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" s="3">
+        <v>44984</v>
+      </c>
+      <c r="B56">
+        <v>0.05</v>
+      </c>
+      <c r="C56" t="s">
+        <v>76</v>
+      </c>
+      <c r="D56" s="3">
+        <v>44986</v>
+      </c>
+      <c r="E56">
+        <v>6.3399999999999998E-2</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57" s="3">
+        <v>44970</v>
+      </c>
+      <c r="B57">
+        <v>0.21</v>
+      </c>
+      <c r="C57" t="s">
+        <v>76</v>
+      </c>
+      <c r="D57" s="3">
+        <v>44972</v>
+      </c>
+      <c r="E57">
+        <v>7.0900000000000005E-2</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58" s="3">
+        <v>44952</v>
+      </c>
+      <c r="B58">
+        <v>0.08</v>
+      </c>
+      <c r="C58" t="s">
+        <v>76</v>
+      </c>
+      <c r="D58" s="3">
+        <v>44956</v>
+      </c>
+      <c r="E58">
+        <v>6.2100000000000002E-2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" s="3">
+        <v>44935</v>
+      </c>
+      <c r="B59">
+        <v>0.02</v>
+      </c>
+      <c r="C59" t="s">
+        <v>76</v>
+      </c>
+      <c r="D59" s="3">
+        <v>44937</v>
+      </c>
+      <c r="E59">
+        <v>7.1499999999999994E-2</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" s="3">
+        <v>44887</v>
+      </c>
+      <c r="B60">
+        <v>0</v>
+      </c>
+      <c r="C60" t="s">
+        <v>76</v>
+      </c>
+      <c r="D60" s="3">
+        <v>44889</v>
+      </c>
+      <c r="E60">
+        <v>7.4399999999999994E-2</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61" s="3">
+        <v>44874</v>
+      </c>
+      <c r="B61">
+        <v>0.05</v>
+      </c>
+      <c r="C61" t="s">
+        <v>76</v>
+      </c>
+      <c r="D61" s="3">
+        <v>44876</v>
+      </c>
+      <c r="E61">
+        <v>7.5600000000000001E-2</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" s="3">
+        <v>44872</v>
+      </c>
+      <c r="B62">
+        <v>0.2</v>
+      </c>
+      <c r="C62" t="s">
+        <v>75</v>
+      </c>
+      <c r="D62" s="3">
+        <v>44874</v>
+      </c>
+      <c r="E62">
+        <v>7.2499999999999995E-2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" s="3">
+        <v>44860</v>
+      </c>
+      <c r="B63">
+        <v>0.04</v>
+      </c>
+      <c r="C63" t="s">
+        <v>76</v>
+      </c>
+      <c r="D63" s="3">
+        <v>44862</v>
+      </c>
+      <c r="E63">
+        <v>6.7699999999999996E-2</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" s="3">
+        <v>44830</v>
+      </c>
+      <c r="B64">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="C64" t="s">
+        <v>75</v>
+      </c>
+      <c r="D64" s="3">
+        <v>44832</v>
+      </c>
+      <c r="E64">
+        <v>7.3599999999999999E-2</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65" s="3">
+        <v>44782</v>
+      </c>
+      <c r="B65">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>75</v>
+      </c>
+      <c r="D65" s="3">
+        <v>44784</v>
+      </c>
+      <c r="E65">
+        <v>7.3700000000000002E-2</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A66" s="3">
+        <v>44778</v>
+      </c>
+      <c r="B66">
+        <v>0.18</v>
+      </c>
+      <c r="C66" t="s">
+        <v>75</v>
+      </c>
+      <c r="D66" s="3">
+        <v>44782</v>
+      </c>
+      <c r="E66">
+        <v>6.9900000000000004E-2</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A67" s="3">
+        <v>44769</v>
+      </c>
+      <c r="B67">
+        <v>0.05</v>
+      </c>
+      <c r="C67" t="s">
+        <v>75</v>
+      </c>
+      <c r="D67" s="3">
+        <v>44771</v>
+      </c>
+      <c r="E67">
+        <v>6.1100000000000002E-2</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A68" s="3">
+        <v>44733</v>
+      </c>
+      <c r="B68">
+        <v>0.05</v>
+      </c>
+      <c r="C68" t="s">
+        <v>76</v>
+      </c>
+      <c r="D68" s="3">
+        <v>44735</v>
+      </c>
+      <c r="E68">
+        <v>7.6399999999999996E-2</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A69" s="3">
+        <v>44708</v>
+      </c>
+      <c r="B69">
+        <v>0.01</v>
+      </c>
+      <c r="C69" t="s">
+        <v>75</v>
+      </c>
+      <c r="D69" s="3">
+        <v>44712</v>
+      </c>
+      <c r="E69">
+        <v>6.8900000000000003E-2</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A70" s="3">
+        <v>44691</v>
+      </c>
+      <c r="B70">
+        <v>0.05</v>
+      </c>
+      <c r="C70" t="s">
+        <v>76</v>
+      </c>
+      <c r="D70" s="3">
+        <v>44693</v>
+      </c>
+      <c r="E70">
+        <v>7.1800000000000003E-2</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A71" s="3">
+        <v>44687</v>
+      </c>
+      <c r="B71">
+        <v>0.18</v>
+      </c>
+      <c r="C71" t="s">
+        <v>75</v>
+      </c>
+      <c r="D71" s="3">
+        <v>44691</v>
+      </c>
+      <c r="E71">
+        <v>6.8400000000000002E-2</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A72" s="3">
+        <v>44678</v>
+      </c>
+      <c r="B72">
+        <v>0.05</v>
+      </c>
+      <c r="C72" t="s">
+        <v>75</v>
+      </c>
+      <c r="D72" s="3">
+        <v>44680</v>
+      </c>
+      <c r="E72">
+        <v>5.7700000000000001E-2</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A73" s="3">
+        <v>44629</v>
+      </c>
+      <c r="B73">
+        <v>0.1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>75</v>
+      </c>
+      <c r="D73" s="3">
+        <v>44631</v>
+      </c>
+      <c r="E73">
+        <v>6.9699999999999998E-2</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A74" s="3">
+        <v>44627</v>
+      </c>
+      <c r="B74">
+        <v>0.08</v>
+      </c>
+      <c r="C74" t="s">
+        <v>75</v>
+      </c>
+      <c r="D74" s="3">
+        <v>44629</v>
+      </c>
+      <c r="E74">
+        <v>6.3100000000000003E-2</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A75" s="3">
+        <v>44603</v>
+      </c>
+      <c r="B75">
+        <v>0.15</v>
+      </c>
+      <c r="C75" t="s">
+        <v>76</v>
+      </c>
+      <c r="D75" s="3">
+        <v>44607</v>
+      </c>
+      <c r="E75">
+        <v>5.7200000000000001E-2</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A76" s="3">
+        <v>44592</v>
+      </c>
+      <c r="B76">
+        <v>0.11</v>
+      </c>
+      <c r="C76" t="s">
+        <v>75</v>
+      </c>
+      <c r="D76" s="3">
+        <v>44594</v>
+      </c>
+      <c r="E76">
+        <v>5.2900000000000003E-2</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A77" s="3">
+        <v>44516</v>
+      </c>
+      <c r="B77">
+        <v>0.06</v>
+      </c>
+      <c r="C77" t="s">
+        <v>76</v>
+      </c>
+      <c r="D77" s="3">
+        <v>44518</v>
+      </c>
+      <c r="E77">
+        <v>4.6399999999999997E-2</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A78" s="3">
+        <v>44509</v>
+      </c>
+      <c r="B78">
+        <v>0.13</v>
+      </c>
+      <c r="C78" t="s">
+        <v>75</v>
+      </c>
+      <c r="D78" s="3">
+        <v>44511</v>
+      </c>
+      <c r="E78">
+        <v>4.2599999999999999E-2</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A79" s="3">
+        <v>44496</v>
+      </c>
+      <c r="B79">
+        <v>0.04</v>
+      </c>
+      <c r="C79" t="s">
+        <v>75</v>
+      </c>
+      <c r="D79" s="3">
+        <v>44498</v>
+      </c>
+      <c r="E79">
+        <v>3.4799999999999998E-2</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A80" s="3">
+        <v>44467</v>
+      </c>
+      <c r="B80">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="C80" t="s">
+        <v>75</v>
+      </c>
+      <c r="D80" s="3">
+        <v>44469</v>
+      </c>
+      <c r="E80">
+        <v>3.1600000000000003E-2</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A81" s="3">
+        <v>44413</v>
+      </c>
+      <c r="B81">
+        <v>0.12</v>
+      </c>
+      <c r="C81" t="s">
+        <v>75</v>
+      </c>
+      <c r="D81" s="3">
+        <v>44417</v>
+      </c>
+      <c r="E81">
+        <v>2.92E-2</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A82" s="3">
+        <v>44412</v>
+      </c>
+      <c r="B82">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="C82" t="s">
+        <v>76</v>
+      </c>
+      <c r="D82" s="3">
+        <v>44414</v>
+      </c>
+      <c r="E82">
+        <v>2.24E-2</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A83" s="3">
+        <v>44405</v>
+      </c>
+      <c r="B83">
+        <v>0.04</v>
+      </c>
+      <c r="C83" t="s">
+        <v>75</v>
+      </c>
+      <c r="D83" s="3">
+        <v>44407</v>
+      </c>
+      <c r="E83">
+        <v>5.5E-2</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A84" s="3">
+        <v>44361</v>
+      </c>
+      <c r="B84">
+        <v>0.05</v>
+      </c>
+      <c r="C84" t="s">
+        <v>75</v>
+      </c>
+      <c r="D84" s="3">
+        <v>44363</v>
+      </c>
+      <c r="E84">
+        <v>6.1499999999999999E-2</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A85" s="3">
+        <v>44328</v>
+      </c>
+      <c r="B85">
+        <v>0.09</v>
+      </c>
+      <c r="C85" t="s">
+        <v>76</v>
+      </c>
+      <c r="D85" s="3">
+        <v>44330</v>
+      </c>
+      <c r="E85">
+        <v>6.5799999999999997E-2</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A86" s="3">
+        <v>44322</v>
+      </c>
+      <c r="B86">
+        <v>0.12</v>
+      </c>
+      <c r="C86" t="s">
+        <v>75</v>
+      </c>
+      <c r="D86" s="3">
+        <v>44326</v>
+      </c>
+      <c r="E86">
+        <v>6.0299999999999999E-2</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A87" s="3">
+        <v>44320</v>
+      </c>
+      <c r="B87">
+        <v>0.04</v>
+      </c>
+      <c r="C87" t="s">
+        <v>75</v>
+      </c>
+      <c r="D87" s="3">
+        <v>44322</v>
+      </c>
+      <c r="E87">
+        <v>5.4600000000000003E-2</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A88" s="3">
+        <v>44272</v>
+      </c>
+      <c r="B88">
+        <v>0.22</v>
+      </c>
+      <c r="C88" t="s">
+        <v>75</v>
+      </c>
+      <c r="D88" s="3">
+        <v>44274</v>
+      </c>
+      <c r="E88">
+        <v>5.6399999999999999E-2</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A89" s="3">
+        <v>44236</v>
+      </c>
+      <c r="B89">
+        <v>0.09</v>
+      </c>
+      <c r="C89" t="s">
+        <v>76</v>
+      </c>
+      <c r="D89" s="3">
+        <v>44238</v>
+      </c>
+      <c r="E89">
+        <v>5.7500000000000002E-2</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A90" s="3">
+        <v>44223</v>
+      </c>
+      <c r="B90">
+        <v>0.05</v>
+      </c>
+      <c r="C90" t="s">
+        <v>76</v>
+      </c>
+      <c r="D90" s="3">
+        <v>44225</v>
+      </c>
+      <c r="E90">
+        <v>5.45E-2</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A91" s="3">
+        <v>44196</v>
+      </c>
+      <c r="B91">
+        <v>0</v>
+      </c>
+      <c r="C91" t="s">
+        <v>76</v>
+      </c>
+      <c r="D91" s="3">
+        <v>44201</v>
+      </c>
+      <c r="E91">
+        <v>6.1800000000000001E-2</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A92" s="3">
+        <v>44174</v>
+      </c>
+      <c r="B92">
+        <v>0</v>
+      </c>
+      <c r="C92" t="s">
+        <v>76</v>
+      </c>
+      <c r="D92" s="3">
+        <v>44176</v>
+      </c>
+      <c r="E92">
+        <v>6.3500000000000001E-2</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A93" s="3">
+        <v>44148</v>
+      </c>
+      <c r="B93">
+        <v>0.05</v>
+      </c>
+      <c r="C93" t="s">
+        <v>76</v>
+      </c>
+      <c r="D93" s="3">
+        <v>44153</v>
+      </c>
+      <c r="E93">
+        <v>7.1099999999999997E-2</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A94" s="3">
+        <v>44144</v>
+      </c>
+      <c r="B94">
+        <v>0.06</v>
+      </c>
+      <c r="C94" t="s">
+        <v>75</v>
+      </c>
+      <c r="D94" s="3">
+        <v>44146</v>
+      </c>
+      <c r="E94">
+        <v>6.6199999999999995E-2</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A95" s="3">
+        <v>44140</v>
+      </c>
+      <c r="B95">
+        <v>0.1</v>
+      </c>
+      <c r="C95" t="s">
+        <v>76</v>
+      </c>
+      <c r="D95" s="3">
+        <v>44144</v>
+      </c>
+      <c r="E95">
+        <v>6.4199999999999993E-2</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A96" s="3">
+        <v>44134</v>
+      </c>
+      <c r="B96">
+        <v>0.03</v>
+      </c>
+      <c r="C96" t="s">
+        <v>75</v>
+      </c>
+      <c r="D96" s="3">
+        <v>44139</v>
+      </c>
+      <c r="E96">
+        <v>5.7799999999999997E-2</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A97" s="3">
+        <v>44106</v>
+      </c>
+      <c r="B97">
+        <v>0</v>
+      </c>
+      <c r="C97" t="s">
+        <v>75</v>
+      </c>
+      <c r="D97" s="3">
+        <v>44110</v>
+      </c>
+      <c r="E97">
+        <v>5.7799999999999997E-2</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A98" s="3">
+        <v>44097</v>
+      </c>
+      <c r="B98">
+        <v>0.05</v>
+      </c>
+      <c r="C98" t="s">
+        <v>76</v>
+      </c>
+      <c r="D98" s="3">
+        <v>44099</v>
+      </c>
+      <c r="E98">
+        <v>5.7500000000000002E-2</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A99" s="3">
+        <v>44055</v>
+      </c>
+      <c r="B99">
+        <v>0.06</v>
+      </c>
+      <c r="C99" t="s">
+        <v>75</v>
+      </c>
+      <c r="D99" s="3">
+        <v>44057</v>
+      </c>
+      <c r="E99">
+        <v>4.9799999999999997E-2</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A100" s="3">
+        <v>44049</v>
+      </c>
+      <c r="B100">
+        <v>0.09</v>
+      </c>
+      <c r="C100" t="s">
+        <v>75</v>
+      </c>
+      <c r="D100" s="3">
+        <v>44053</v>
+      </c>
+      <c r="E100">
+        <v>4.65E-2</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A101" s="3">
+        <v>44039</v>
+      </c>
+      <c r="B101">
+        <v>0.03</v>
+      </c>
+      <c r="C101" t="s">
+        <v>75</v>
+      </c>
+      <c r="D101" s="3">
+        <v>44041</v>
+      </c>
+      <c r="E101">
+        <v>4.24E-2</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A102" s="3">
+        <v>44007</v>
+      </c>
+      <c r="B102">
+        <v>0.09</v>
+      </c>
+      <c r="C102" t="s">
+        <v>76</v>
+      </c>
+      <c r="D102" s="3">
+        <v>44011</v>
+      </c>
+      <c r="E102">
+        <v>3.9699999999999999E-2</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A103" s="3">
+        <v>43993</v>
+      </c>
+      <c r="B103">
+        <v>0.05</v>
+      </c>
+      <c r="C103" t="s">
+        <v>76</v>
+      </c>
+      <c r="D103" s="3">
+        <v>43997</v>
+      </c>
+      <c r="E103">
+        <v>8.9399999999999993E-2</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A104" s="3">
+        <v>43963</v>
+      </c>
+      <c r="B104">
+        <v>0.12</v>
+      </c>
+      <c r="C104" t="s">
+        <v>75</v>
+      </c>
+      <c r="D104" s="3">
+        <v>43965</v>
+      </c>
+      <c r="E104">
+        <v>8.7599999999999997E-2</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A105" s="3">
+        <v>43901</v>
+      </c>
+      <c r="B105">
+        <v>0.15</v>
+      </c>
+      <c r="C105" t="s">
+        <v>75</v>
+      </c>
+      <c r="D105" s="3">
+        <v>43903</v>
+      </c>
+      <c r="E105">
+        <v>7.4399999999999994E-2</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A106" s="3">
+        <v>43895</v>
+      </c>
+      <c r="B106">
+        <v>0.06</v>
+      </c>
+      <c r="C106" t="s">
+        <v>75</v>
+      </c>
+      <c r="D106" s="3">
+        <v>43899</v>
+      </c>
+      <c r="E106">
+        <v>6.8699999999999997E-2</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A107" s="3">
+        <v>43871</v>
+      </c>
+      <c r="B107">
+        <v>0.1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>75</v>
+      </c>
+      <c r="D107" s="3">
+        <v>43873</v>
+      </c>
+      <c r="E107">
+        <v>7.9000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A108" s="3">
+        <v>43866</v>
+      </c>
+      <c r="B108">
+        <v>0.04</v>
+      </c>
+      <c r="C108" t="s">
+        <v>76</v>
+      </c>
+      <c r="D108" s="3">
+        <v>43868</v>
+      </c>
+      <c r="E108">
+        <v>7.51E-2</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A109" s="3">
+        <v>43858</v>
+      </c>
+      <c r="B109">
+        <v>0.05</v>
+      </c>
+      <c r="C109" t="s">
+        <v>75</v>
+      </c>
+      <c r="D109" s="3">
+        <v>43860</v>
+      </c>
+      <c r="E109">
+        <v>7.0300000000000001E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A3310AA-E392-493A-A2AE-BF420C7EE2F4}">
   <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2217,7 +4448,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D64E9A49-6EF8-4D39-B285-D1831FBA55F5}">
   <dimension ref="A1:E26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2676,7 +4907,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7080F36D-9347-419F-84A7-BD01AB3CDA0E}">
   <dimension ref="A1:E27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3151,7 +5382,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46F89605-F7C1-48CA-8476-6F366E15000B}">
   <dimension ref="A1:E62"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4220,7 +6451,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2920B5B7-5BAB-44A1-8A1D-9FB19177ABE2}">
   <dimension ref="A1:E23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4627,7 +6858,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B54206EA-71E2-4EF2-8BA5-37630DBAD1A4}">
   <dimension ref="A1:E27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5099,361 +7330,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{200EB5CF-E323-4820-B096-9F8315944A3A}">
-  <dimension ref="A1:E20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.5703125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>72</v>
-      </c>
-      <c r="B2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D2" t="s">
-        <v>79</v>
-      </c>
-      <c r="E2" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="3">
-        <v>45791</v>
-      </c>
-      <c r="B3">
-        <v>0.32</v>
-      </c>
-      <c r="C3" t="s">
-        <v>74</v>
-      </c>
-      <c r="D3" s="3">
-        <v>45792</v>
-      </c>
-      <c r="E3">
-        <v>9.0499999999999997E-2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="3">
-        <v>45728</v>
-      </c>
-      <c r="B4">
-        <v>0.12</v>
-      </c>
-      <c r="C4" t="s">
-        <v>74</v>
-      </c>
-      <c r="D4" s="3">
-        <v>45729</v>
-      </c>
-      <c r="E4">
-        <v>3.7400000000000003E-2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="3">
-        <v>45616</v>
-      </c>
-      <c r="B5">
-        <v>0.4</v>
-      </c>
-      <c r="C5" t="s">
-        <v>74</v>
-      </c>
-      <c r="D5" s="3">
-        <v>45617</v>
-      </c>
-      <c r="E5">
-        <v>9.6199999999999994E-2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="3">
-        <v>45518</v>
-      </c>
-      <c r="B6">
-        <v>0.33</v>
-      </c>
-      <c r="C6" t="s">
-        <v>74</v>
-      </c>
-      <c r="D6" s="3">
-        <v>45519</v>
-      </c>
-      <c r="E6">
-        <v>7.9600000000000004E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="3">
-        <v>45426</v>
-      </c>
-      <c r="B7">
-        <v>0.36</v>
-      </c>
-      <c r="C7" t="s">
-        <v>74</v>
-      </c>
-      <c r="D7" s="3">
-        <v>45428</v>
-      </c>
-      <c r="E7">
-        <v>8.6099999999999996E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="3">
-        <v>45357</v>
-      </c>
-      <c r="B8">
-        <v>0.5</v>
-      </c>
-      <c r="C8" t="s">
-        <v>74</v>
-      </c>
-      <c r="D8" s="3">
-        <v>45359</v>
-      </c>
-      <c r="E8">
-        <v>0.1246</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="3">
-        <v>45244</v>
-      </c>
-      <c r="B9">
-        <v>0.68</v>
-      </c>
-      <c r="C9" t="s">
-        <v>74</v>
-      </c>
-      <c r="D9" s="3">
-        <v>45246</v>
-      </c>
-      <c r="E9">
-        <v>0.15920000000000001</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="3">
-        <v>45153</v>
-      </c>
-      <c r="B10">
-        <v>0.48</v>
-      </c>
-      <c r="C10" t="s">
-        <v>74</v>
-      </c>
-      <c r="D10" s="3">
-        <v>45155</v>
-      </c>
-      <c r="E10">
-        <v>0.1106</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="3">
-        <v>45062</v>
-      </c>
-      <c r="B11">
-        <v>0.26</v>
-      </c>
-      <c r="C11" t="s">
-        <v>74</v>
-      </c>
-      <c r="D11" s="3">
-        <v>45064</v>
-      </c>
-      <c r="E11">
-        <v>6.0699999999999997E-2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="3">
-        <v>44999</v>
-      </c>
-      <c r="B12">
-        <v>0.62</v>
-      </c>
-      <c r="C12" t="s">
-        <v>74</v>
-      </c>
-      <c r="D12" s="3">
-        <v>45001</v>
-      </c>
-      <c r="E12">
-        <v>0.14480000000000001</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="3">
-        <v>44880</v>
-      </c>
-      <c r="B13">
-        <v>0.47</v>
-      </c>
-      <c r="C13" t="s">
-        <v>74</v>
-      </c>
-      <c r="D13" s="3">
-        <v>44882</v>
-      </c>
-      <c r="E13">
-        <v>0.1014</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="3">
-        <v>44789</v>
-      </c>
-      <c r="B14">
-        <v>0.71</v>
-      </c>
-      <c r="C14" t="s">
-        <v>74</v>
-      </c>
-      <c r="D14" s="3">
-        <v>44791</v>
-      </c>
-      <c r="E14">
-        <v>0.1512</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="3">
-        <v>44698</v>
-      </c>
-      <c r="B15">
-        <v>0.47</v>
-      </c>
-      <c r="C15" t="s">
-        <v>74</v>
-      </c>
-      <c r="D15" s="3">
-        <v>44700</v>
-      </c>
-      <c r="E15">
-        <v>9.69E-2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="3">
-        <v>44271</v>
-      </c>
-      <c r="B16">
-        <v>0.28000000000000003</v>
-      </c>
-      <c r="C16" t="s">
-        <v>74</v>
-      </c>
-      <c r="D16" s="3">
-        <v>44273</v>
-      </c>
-      <c r="E16">
-        <v>5.6500000000000002E-2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="3">
-        <v>44152</v>
-      </c>
-      <c r="B17">
-        <v>0.34</v>
-      </c>
-      <c r="C17" t="s">
-        <v>74</v>
-      </c>
-      <c r="D17" s="3">
-        <v>44154</v>
-      </c>
-      <c r="E17">
-        <v>7.5300000000000006E-2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="3">
-        <v>44061</v>
-      </c>
-      <c r="B18">
-        <v>0.39</v>
-      </c>
-      <c r="C18" t="s">
-        <v>74</v>
-      </c>
-      <c r="D18" s="3">
-        <v>44063</v>
-      </c>
-      <c r="E18">
-        <v>8.7800000000000003E-2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="3">
-        <v>43970</v>
-      </c>
-      <c r="B19">
-        <v>0.46</v>
-      </c>
-      <c r="C19" t="s">
-        <v>74</v>
-      </c>
-      <c r="D19" s="3">
-        <v>43972</v>
-      </c>
-      <c r="E19">
-        <v>0.11509999999999999</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="3">
-        <v>43909</v>
-      </c>
-      <c r="B20">
-        <v>0.11</v>
-      </c>
-      <c r="C20" t="s">
-        <v>74</v>
-      </c>
-      <c r="D20" s="3">
-        <v>43913</v>
-      </c>
-      <c r="E20">
-        <v>2.53E-2</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
No tengo claro que tanto cambien en las hojas
</commit_message>
<xml_diff>
--- a/Historico de Fibras.xlsx
+++ b/Historico de Fibras.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\M R\Documents\Python\BDHistorico\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CEA67E4-FA16-4084-A307-3A44AACBBFDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F1CCCA5C-0C2A-4A81-B0BE-6E2F04E053C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="15600" windowHeight="19440" tabRatio="705" activeTab="2" xr2:uid="{61FC1FF2-927D-4FA9-8C22-EC769C0CC026}"/>
+    <workbookView xWindow="-13620" yWindow="-120" windowWidth="13740" windowHeight="21840" tabRatio="705" xr2:uid="{61FC1FF2-927D-4FA9-8C22-EC769C0CC026}"/>
   </bookViews>
   <sheets>
     <sheet name="Fechas de distribucion" sheetId="1" r:id="rId1"/>
@@ -19,13 +19,14 @@
     <sheet name="FIHO12" sheetId="7" r:id="rId4"/>
     <sheet name="FIBRAPL14" sheetId="2" r:id="rId5"/>
     <sheet name="FUNO11" sheetId="3" r:id="rId6"/>
-    <sheet name="FMTY14" sheetId="4" r:id="rId7"/>
-    <sheet name="FNOVA17" sheetId="10" r:id="rId8"/>
-    <sheet name="FIBRAMQ12" sheetId="5" r:id="rId9"/>
+    <sheet name="FIBRAMQ12" sheetId="5" r:id="rId7"/>
+    <sheet name="FMTY14" sheetId="4" r:id="rId8"/>
+    <sheet name="FNOVA17" sheetId="10" r:id="rId9"/>
     <sheet name="FHIPO14" sheetId="6" r:id="rId10"/>
     <sheet name="DANHOS13" sheetId="8" r:id="rId11"/>
   </sheets>
   <calcPr calcId="181029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="579" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="589" uniqueCount="87">
   <si>
     <t>ENERO</t>
   </si>
@@ -696,7 +697,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24B1044F-9D4D-44C5-B1E7-5FBBB32197E2}">
-  <dimension ref="A1:J53"/>
+  <dimension ref="A1:J55"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="17.28515625" bestFit="1" customWidth="1"/>
@@ -1236,6 +1237,18 @@
       <c r="D39" s="7">
         <v>1732468.6783080092</v>
       </c>
+      <c r="E39" t="s">
+        <v>4</v>
+      </c>
+      <c r="F39" t="s">
+        <v>6</v>
+      </c>
+      <c r="G39" t="s">
+        <v>9</v>
+      </c>
+      <c r="H39" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C40" t="s">
@@ -1378,6 +1391,28 @@
       </c>
       <c r="G53" t="s">
         <v>70</v>
+      </c>
+    </row>
+    <row r="54" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C54" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D54" t="s">
+        <v>4</v>
+      </c>
+      <c r="E54" t="s">
+        <v>6</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+      <c r="G54" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="55" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C55" s="5" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -5383,8 +5418,8 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46F89605-F7C1-48CA-8476-6F366E15000B}">
-  <dimension ref="A1:E62"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B54206EA-71E2-4EF2-8BA5-37630DBAD1A4}">
+  <dimension ref="A1:E27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.7109375" bestFit="1" customWidth="1"/>
@@ -5394,19 +5429,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>14</v>
+        <v>82</v>
       </c>
       <c r="B1" t="s">
-        <v>14</v>
+        <v>82</v>
       </c>
       <c r="C1" t="s">
-        <v>14</v>
+        <v>82</v>
       </c>
       <c r="D1" t="s">
-        <v>14</v>
+        <v>82</v>
       </c>
       <c r="E1" t="s">
-        <v>14</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -5428,1022 +5463,427 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
-        <v>45868</v>
+        <v>45834</v>
       </c>
       <c r="B3">
-        <v>0.09</v>
+        <v>0.61</v>
       </c>
       <c r="C3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D3" s="3">
-        <v>45869</v>
+        <v>45835</v>
       </c>
       <c r="E3">
-        <v>7.5700000000000003E-2</v>
+        <v>7.9500000000000001E-2</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
-        <v>45841</v>
+        <v>45728</v>
       </c>
       <c r="B4">
-        <v>0.09</v>
+        <v>0.53</v>
       </c>
       <c r="C4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D4" s="3">
-        <v>45842</v>
+        <v>45729</v>
       </c>
       <c r="E4">
-        <v>7.6799999999999993E-2</v>
+        <v>6.83E-2</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
-        <v>45806</v>
+        <v>45686</v>
       </c>
       <c r="B5">
-        <v>0.09</v>
+        <v>0.53</v>
       </c>
       <c r="C5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D5" s="3">
-        <v>45807</v>
+        <v>45687</v>
       </c>
       <c r="E5">
-        <v>7.1900000000000006E-2</v>
+        <v>6.5100000000000005E-2</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
-        <v>45776</v>
+        <v>45561</v>
       </c>
       <c r="B6">
-        <v>0.09</v>
+        <v>0.53</v>
       </c>
       <c r="C6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D6" s="3">
-        <v>45777</v>
+        <v>45562</v>
       </c>
       <c r="E6">
-        <v>7.4300000000000005E-2</v>
+        <v>6.6100000000000006E-2</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
-        <v>45727</v>
+        <v>45457</v>
       </c>
       <c r="B7">
-        <v>0.09</v>
+        <v>0.53</v>
       </c>
       <c r="C7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D7" s="3">
-        <v>45728</v>
+        <v>45460</v>
       </c>
       <c r="E7">
-        <v>7.3899999999999993E-2</v>
+        <v>6.83E-2</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
-        <v>45715</v>
+        <v>45363</v>
       </c>
       <c r="B8">
-        <v>0.09</v>
+        <v>0.68</v>
       </c>
       <c r="C8" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="D8" s="3">
-        <v>45716</v>
+        <v>45365</v>
       </c>
       <c r="E8">
-        <v>6.6699999999999995E-2</v>
+        <v>8.0500000000000002E-2</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
-        <v>45687</v>
+        <v>45357</v>
       </c>
       <c r="B9">
-        <v>0.09</v>
+        <v>0.53</v>
       </c>
       <c r="C9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D9" s="3">
-        <v>45688</v>
+        <v>45359</v>
       </c>
       <c r="E9">
-        <v>8.8900000000000007E-2</v>
+        <v>6.0299999999999999E-2</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
-        <v>45652</v>
+        <v>45317</v>
       </c>
       <c r="B10">
-        <v>0.08</v>
+        <v>0.53</v>
       </c>
       <c r="C10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D10" s="3">
-        <v>45653</v>
+        <v>45321</v>
       </c>
       <c r="E10">
-        <v>8.8300000000000003E-2</v>
+        <v>6.2600000000000003E-2</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
-        <v>45624</v>
+        <v>45195</v>
       </c>
       <c r="B11">
-        <v>0.08</v>
+        <v>0.53</v>
       </c>
       <c r="C11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D11" s="3">
-        <v>45625</v>
+        <v>45197</v>
       </c>
       <c r="E11">
-        <v>9.1399999999999995E-2</v>
+        <v>6.8599999999999994E-2</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
-        <v>45595</v>
+        <v>45091</v>
       </c>
       <c r="B12">
-        <v>0.08</v>
+        <v>0.53</v>
       </c>
       <c r="C12" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D12" s="3">
-        <v>45596</v>
+        <v>45093</v>
       </c>
       <c r="E12">
-        <v>8.8200000000000001E-2</v>
+        <v>7.0099999999999996E-2</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
-        <v>45562</v>
+        <v>44993</v>
       </c>
       <c r="B13">
-        <v>0.08</v>
+        <v>0.88</v>
       </c>
       <c r="C13" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="D13" s="3">
-        <v>45565</v>
+        <v>44995</v>
       </c>
       <c r="E13">
-        <v>8.9899999999999994E-2</v>
+        <v>9.3700000000000006E-2</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
-        <v>45533</v>
+        <v>44986</v>
       </c>
       <c r="B14">
-        <v>0.08</v>
+        <v>0.5</v>
       </c>
       <c r="C14" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D14" s="3">
-        <v>45534</v>
+        <v>44988</v>
       </c>
       <c r="E14">
-        <v>9.1899999999999996E-2</v>
+        <v>6.3700000000000007E-2</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
-        <v>45503</v>
+        <v>44952</v>
       </c>
       <c r="B15">
-        <v>0.08</v>
+        <v>0.5</v>
       </c>
       <c r="C15" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D15" s="3">
-        <v>45504</v>
+        <v>44956</v>
       </c>
       <c r="E15">
-        <v>9.74E-2</v>
+        <v>6.4000000000000001E-2</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
-        <v>45470</v>
+        <v>44830</v>
       </c>
       <c r="B16">
-        <v>7.0000000000000007E-2</v>
+        <v>0.5</v>
       </c>
       <c r="C16" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D16" s="3">
-        <v>45471</v>
+        <v>44832</v>
       </c>
       <c r="E16">
-        <v>9.2200000000000004E-2</v>
+        <v>7.8200000000000006E-2</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
-        <v>45351</v>
+        <v>44726</v>
       </c>
       <c r="B17">
-        <v>0.23</v>
+        <v>0.5</v>
       </c>
       <c r="C17" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D17" s="3">
-        <v>45355</v>
+        <v>44728</v>
       </c>
       <c r="E17">
-        <v>7.0499999999999993E-2</v>
+        <v>8.2000000000000003E-2</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
-        <v>45349</v>
+        <v>44629</v>
       </c>
       <c r="B18">
-        <v>0.08</v>
+        <v>0.48</v>
       </c>
       <c r="C18" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D18" s="3">
-        <v>45351</v>
+        <v>44631</v>
       </c>
       <c r="E18">
-        <v>5.11E-2</v>
+        <v>7.9600000000000004E-2</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
-        <v>45320</v>
+        <v>44587</v>
       </c>
       <c r="B19">
-        <v>0.08</v>
+        <v>0.48</v>
       </c>
       <c r="C19" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D19" s="3">
-        <v>45322</v>
+        <v>44589</v>
       </c>
       <c r="E19">
-        <v>4.4200000000000003E-2</v>
+        <v>7.9699999999999993E-2</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
-        <v>45287</v>
+        <v>44462</v>
       </c>
       <c r="B20">
-        <v>0.08</v>
+        <v>0.48</v>
       </c>
       <c r="C20" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D20" s="3">
-        <v>45289</v>
+        <v>44466</v>
       </c>
       <c r="E20">
-        <v>3.7999999999999999E-2</v>
+        <v>7.3599999999999999E-2</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
-        <v>45258</v>
+        <v>44358</v>
       </c>
       <c r="B21">
-        <v>0.08</v>
+        <v>0.48</v>
       </c>
       <c r="C21" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D21" s="3">
-        <v>45260</v>
+        <v>44362</v>
       </c>
       <c r="E21">
-        <v>3.4599999999999999E-2</v>
+        <v>8.0600000000000005E-2</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
-        <v>45226</v>
+        <v>44265</v>
       </c>
       <c r="B22">
-        <v>0.08</v>
+        <v>0.48</v>
       </c>
       <c r="C22" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D22" s="3">
-        <v>45230</v>
+        <v>44267</v>
       </c>
       <c r="E22">
-        <v>2.8899999999999999E-2</v>
+        <v>7.4200000000000002E-2</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
-        <v>45196</v>
+        <v>44222</v>
       </c>
       <c r="B23">
-        <v>7.0000000000000007E-2</v>
+        <v>0.47</v>
       </c>
       <c r="C23" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D23" s="3">
-        <v>45198</v>
+        <v>44224</v>
       </c>
       <c r="E23">
-        <v>9.2700000000000005E-2</v>
+        <v>6.7599999999999993E-2</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
-        <v>45167</v>
+        <v>44097</v>
       </c>
       <c r="B24">
-        <v>7.0000000000000007E-2</v>
+        <v>0.48</v>
       </c>
       <c r="C24" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D24" s="3">
-        <v>45169</v>
+        <v>44099</v>
       </c>
       <c r="E24">
-        <v>8.1299999999999997E-2</v>
+        <v>7.5800000000000006E-2</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
-        <v>45134</v>
+        <v>43992</v>
       </c>
       <c r="B25">
-        <v>7.0000000000000007E-2</v>
+        <v>0.48</v>
       </c>
       <c r="C25" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D25" s="3">
-        <v>45138</v>
+        <v>43994</v>
       </c>
       <c r="E25">
-        <v>8.7900000000000006E-2</v>
+        <v>7.8299999999999995E-2</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="3">
-        <v>45014</v>
+        <v>43899</v>
       </c>
       <c r="B26">
-        <v>0.09</v>
+        <v>0.45</v>
       </c>
       <c r="C26" t="s">
         <v>75</v>
       </c>
       <c r="D26" s="3">
-        <v>45016</v>
+        <v>43901</v>
       </c>
       <c r="E26">
-        <v>0.1032</v>
+        <v>6.54E-2</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="3">
-        <v>44979</v>
+        <v>43852</v>
       </c>
       <c r="B27">
-        <v>0.34</v>
+        <v>0.46</v>
       </c>
       <c r="C27" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D27" s="3">
-        <v>44981</v>
+        <v>43854</v>
       </c>
       <c r="E27">
-        <v>9.4600000000000004E-2</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="3">
-        <v>44953</v>
-      </c>
-      <c r="B28">
-        <v>0.09</v>
-      </c>
-      <c r="C28" t="s">
-        <v>76</v>
-      </c>
-      <c r="D28" s="3">
-        <v>44957</v>
-      </c>
-      <c r="E28">
-        <v>8.1000000000000003E-2</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="3">
-        <v>44923</v>
-      </c>
-      <c r="B29">
-        <v>0.08</v>
-      </c>
-      <c r="C29" t="s">
-        <v>75</v>
-      </c>
-      <c r="D29" s="3">
-        <v>44925</v>
-      </c>
-      <c r="E29">
-        <v>7.8600000000000003E-2</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" s="3">
-        <v>44893</v>
-      </c>
-      <c r="B30">
-        <v>0.08</v>
-      </c>
-      <c r="C30" t="s">
-        <v>75</v>
-      </c>
-      <c r="D30" s="3">
-        <v>44895</v>
-      </c>
-      <c r="E30">
-        <v>8.0600000000000005E-2</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="3">
-        <v>44861</v>
-      </c>
-      <c r="B31">
-        <v>0.08</v>
-      </c>
-      <c r="C31" t="s">
-        <v>75</v>
-      </c>
-      <c r="D31" s="3">
-        <v>44865</v>
-      </c>
-      <c r="E31">
-        <v>8.0199999999999994E-2</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="3">
-        <v>44812</v>
-      </c>
-      <c r="B32">
-        <v>0.08</v>
-      </c>
-      <c r="C32" t="s">
-        <v>75</v>
-      </c>
-      <c r="D32" s="3">
-        <v>44816</v>
-      </c>
-      <c r="E32">
-        <v>8.5400000000000004E-2</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="3">
-        <v>44802</v>
-      </c>
-      <c r="B33">
-        <v>0.08</v>
-      </c>
-      <c r="C33" t="s">
-        <v>75</v>
-      </c>
-      <c r="D33" s="3">
-        <v>44804</v>
-      </c>
-      <c r="E33">
-        <v>7.8700000000000006E-2</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="3">
-        <v>44769</v>
-      </c>
-      <c r="B34">
-        <v>0.08</v>
-      </c>
-      <c r="C34" t="s">
-        <v>75</v>
-      </c>
-      <c r="D34" s="3">
-        <v>44771</v>
-      </c>
-      <c r="E34">
-        <v>7.8200000000000006E-2</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="3">
-        <v>44740</v>
-      </c>
-      <c r="B35">
-        <v>0.08</v>
-      </c>
-      <c r="C35" t="s">
-        <v>75</v>
-      </c>
-      <c r="D35" s="3">
-        <v>44742</v>
-      </c>
-      <c r="E35">
-        <v>7.7100000000000002E-2</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="3">
-        <v>44708</v>
-      </c>
-      <c r="B36">
-        <v>0.08</v>
-      </c>
-      <c r="C36" t="s">
-        <v>75</v>
-      </c>
-      <c r="D36" s="3">
-        <v>44712</v>
-      </c>
-      <c r="E36">
-        <v>6.9500000000000006E-2</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" s="3">
-        <v>44678</v>
-      </c>
-      <c r="B37">
-        <v>0.08</v>
-      </c>
-      <c r="C37" t="s">
-        <v>75</v>
-      </c>
-      <c r="D37" s="3">
-        <v>44680</v>
-      </c>
-      <c r="E37">
-        <v>6.0999999999999999E-2</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="3">
-        <v>44629</v>
-      </c>
-      <c r="B38">
-        <v>0.08</v>
-      </c>
-      <c r="C38" t="s">
-        <v>75</v>
-      </c>
-      <c r="D38" s="3">
-        <v>44631</v>
-      </c>
-      <c r="E38">
-        <v>5.6300000000000003E-2</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="3">
-        <v>44616</v>
-      </c>
-      <c r="B39">
-        <v>0.08</v>
-      </c>
-      <c r="C39" t="s">
-        <v>75</v>
-      </c>
-      <c r="D39" s="3">
-        <v>44620</v>
-      </c>
-      <c r="E39">
-        <v>4.8800000000000003E-2</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" s="3">
-        <v>44588</v>
-      </c>
-      <c r="B40">
-        <v>0.08</v>
-      </c>
-      <c r="C40" t="s">
-        <v>75</v>
-      </c>
-      <c r="D40" s="3">
-        <v>44592</v>
-      </c>
-      <c r="E40">
-        <v>4.2099999999999999E-2</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" s="3">
-        <v>44559</v>
-      </c>
-      <c r="B41">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="C41" t="s">
-        <v>75</v>
-      </c>
-      <c r="D41" s="3">
-        <v>44561</v>
-      </c>
-      <c r="E41">
-        <v>3.5999999999999997E-2</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" s="3">
-        <v>44526</v>
-      </c>
-      <c r="B42">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="C42" t="s">
-        <v>75</v>
-      </c>
-      <c r="D42" s="3">
-        <v>44530</v>
-      </c>
-      <c r="E42">
-        <v>3.0200000000000001E-2</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" s="3">
-        <v>44496</v>
-      </c>
-      <c r="B43">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="C43" t="s">
-        <v>75</v>
-      </c>
-      <c r="D43" s="3">
-        <v>44498</v>
-      </c>
-      <c r="E43">
-        <v>7.6399999999999996E-2</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" s="3">
-        <v>44467</v>
-      </c>
-      <c r="B44">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="C44" t="s">
-        <v>76</v>
-      </c>
-      <c r="D44" s="3">
-        <v>44469</v>
-      </c>
-      <c r="E44">
-        <v>7.7700000000000005E-2</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" s="3">
-        <v>44435</v>
-      </c>
-      <c r="B45">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="C45" t="s">
-        <v>76</v>
-      </c>
-      <c r="D45" s="3">
-        <v>44439</v>
-      </c>
-      <c r="E45">
-        <v>7.9500000000000001E-2</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" s="3">
-        <v>44405</v>
-      </c>
-      <c r="B46">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="C46" t="s">
-        <v>76</v>
-      </c>
-      <c r="D46" s="3">
-        <v>44407</v>
-      </c>
-      <c r="E46">
-        <v>8.1699999999999995E-2</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A47" s="3">
-        <v>44375</v>
-      </c>
-      <c r="B47">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="C47" t="s">
-        <v>75</v>
-      </c>
-      <c r="D47" s="3">
-        <v>44377</v>
-      </c>
-      <c r="E47">
-        <v>8.0299999999999996E-2</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" s="3">
-        <v>44343</v>
-      </c>
-      <c r="B48">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="C48" t="s">
-        <v>75</v>
-      </c>
-      <c r="D48" s="3">
-        <v>44347</v>
-      </c>
-      <c r="E48">
-        <v>8.6900000000000005E-2</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A49" s="3">
-        <v>44314</v>
-      </c>
-      <c r="B49">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="C49" t="s">
-        <v>75</v>
-      </c>
-      <c r="D49" s="3">
-        <v>44316</v>
-      </c>
-      <c r="E49">
-        <v>8.8999999999999996E-2</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" s="3">
-        <v>44265</v>
-      </c>
-      <c r="B50">
-        <v>0.08</v>
-      </c>
-      <c r="C50" t="s">
-        <v>75</v>
-      </c>
-      <c r="D50" s="3">
-        <v>44267</v>
-      </c>
-      <c r="E50">
-        <v>9.2100000000000001E-2</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" s="3">
-        <v>44251</v>
-      </c>
-      <c r="B51">
-        <v>0.08</v>
-      </c>
-      <c r="C51" t="s">
-        <v>75</v>
-      </c>
-      <c r="D51" s="3">
-        <v>44253</v>
-      </c>
-      <c r="E51">
-        <v>8.3199999999999996E-2</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" s="3">
-        <v>44223</v>
-      </c>
-      <c r="B52">
-        <v>0.08</v>
-      </c>
-      <c r="C52" t="s">
-        <v>75</v>
-      </c>
-      <c r="D52" s="3">
-        <v>44225</v>
-      </c>
-      <c r="E52">
-        <v>9.4200000000000006E-2</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" s="3">
-        <v>44194</v>
-      </c>
-      <c r="B53">
-        <v>0.09</v>
-      </c>
-      <c r="C53" t="s">
-        <v>75</v>
-      </c>
-      <c r="D53" s="3">
-        <v>44196</v>
-      </c>
-      <c r="E53">
-        <v>8.5000000000000006E-2</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" s="3">
-        <v>44161</v>
-      </c>
-      <c r="B54">
-        <v>0.09</v>
-      </c>
-      <c r="C54" t="s">
-        <v>75</v>
-      </c>
-      <c r="D54" s="3">
-        <v>44165</v>
-      </c>
-      <c r="E54">
-        <v>7.6399999999999996E-2</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A55" s="3">
-        <v>44132</v>
-      </c>
-      <c r="B55">
-        <v>0.09</v>
-      </c>
-      <c r="C55" t="s">
-        <v>75</v>
-      </c>
-      <c r="D55" s="3">
-        <v>44134</v>
-      </c>
-      <c r="E55">
-        <v>7.8100000000000003E-2</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A56" s="3">
-        <v>44102</v>
-      </c>
-      <c r="B56">
-        <v>0.09</v>
-      </c>
-      <c r="C56" t="s">
-        <v>75</v>
-      </c>
-      <c r="D56" s="3">
-        <v>44104</v>
-      </c>
-      <c r="E56">
-        <v>7.22E-2</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A57" s="3">
-        <v>44070</v>
-      </c>
-      <c r="B57">
-        <v>0.09</v>
-      </c>
-      <c r="C57" t="s">
-        <v>75</v>
-      </c>
-      <c r="D57" s="3">
-        <v>44074</v>
-      </c>
-      <c r="E57">
-        <v>9.3100000000000002E-2</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A58" s="3">
-        <v>44041</v>
-      </c>
-      <c r="B58">
-        <v>0.09</v>
-      </c>
-      <c r="C58" t="s">
-        <v>75</v>
-      </c>
-      <c r="D58" s="3">
-        <v>44043</v>
-      </c>
-      <c r="E58">
-        <v>8.3299999999999999E-2</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A59" s="3">
-        <v>44008</v>
-      </c>
-      <c r="B59">
-        <v>0.09</v>
-      </c>
-      <c r="C59" t="s">
-        <v>75</v>
-      </c>
-      <c r="D59" s="3">
-        <v>44012</v>
-      </c>
-      <c r="E59">
-        <v>0.104</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A60" s="3">
-        <v>43978</v>
-      </c>
-      <c r="B60">
-        <v>0.09</v>
-      </c>
-      <c r="C60" t="s">
-        <v>75</v>
-      </c>
-      <c r="D60" s="3">
-        <v>43980</v>
-      </c>
-      <c r="E60">
-        <v>9.1399999999999995E-2</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A61" s="3">
-        <v>43949</v>
-      </c>
-      <c r="B61">
-        <v>0.09</v>
-      </c>
-      <c r="C61" t="s">
-        <v>75</v>
-      </c>
-      <c r="D61" s="3">
-        <v>43951</v>
-      </c>
-      <c r="E61">
-        <v>9.2399999999999996E-2</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A62" s="3">
-        <v>43882</v>
-      </c>
-      <c r="B62">
-        <v>0.17</v>
-      </c>
-      <c r="C62" t="s">
-        <v>75</v>
-      </c>
-      <c r="D62" s="3">
-        <v>43886</v>
-      </c>
-      <c r="E62">
-        <v>6.4699999999999994E-2</v>
+        <v>6.3399999999999998E-2</v>
       </c>
     </row>
   </sheetData>
@@ -6452,6 +5892,1076 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46F89605-F7C1-48CA-8476-6F366E15000B}">
+  <dimension ref="A1:E62"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D2" t="s">
+        <v>79</v>
+      </c>
+      <c r="E2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="3">
+        <v>45868</v>
+      </c>
+      <c r="B3">
+        <v>0.09</v>
+      </c>
+      <c r="C3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D3" s="3">
+        <v>45869</v>
+      </c>
+      <c r="E3">
+        <v>7.5700000000000003E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="3">
+        <v>45841</v>
+      </c>
+      <c r="B4">
+        <v>0.09</v>
+      </c>
+      <c r="C4" t="s">
+        <v>75</v>
+      </c>
+      <c r="D4" s="3">
+        <v>45842</v>
+      </c>
+      <c r="E4">
+        <v>7.6799999999999993E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="3">
+        <v>45806</v>
+      </c>
+      <c r="B5">
+        <v>0.09</v>
+      </c>
+      <c r="C5" t="s">
+        <v>75</v>
+      </c>
+      <c r="D5" s="3">
+        <v>45807</v>
+      </c>
+      <c r="E5">
+        <v>7.1900000000000006E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="3">
+        <v>45776</v>
+      </c>
+      <c r="B6">
+        <v>0.09</v>
+      </c>
+      <c r="C6" t="s">
+        <v>75</v>
+      </c>
+      <c r="D6" s="3">
+        <v>45777</v>
+      </c>
+      <c r="E6">
+        <v>7.4300000000000005E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="3">
+        <v>45727</v>
+      </c>
+      <c r="B7">
+        <v>0.09</v>
+      </c>
+      <c r="C7" t="s">
+        <v>75</v>
+      </c>
+      <c r="D7" s="3">
+        <v>45728</v>
+      </c>
+      <c r="E7">
+        <v>7.3899999999999993E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="3">
+        <v>45715</v>
+      </c>
+      <c r="B8">
+        <v>0.09</v>
+      </c>
+      <c r="C8" t="s">
+        <v>75</v>
+      </c>
+      <c r="D8" s="3">
+        <v>45716</v>
+      </c>
+      <c r="E8">
+        <v>6.6699999999999995E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="3">
+        <v>45687</v>
+      </c>
+      <c r="B9">
+        <v>0.09</v>
+      </c>
+      <c r="C9" t="s">
+        <v>75</v>
+      </c>
+      <c r="D9" s="3">
+        <v>45688</v>
+      </c>
+      <c r="E9">
+        <v>8.8900000000000007E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="3">
+        <v>45652</v>
+      </c>
+      <c r="B10">
+        <v>0.08</v>
+      </c>
+      <c r="C10" t="s">
+        <v>75</v>
+      </c>
+      <c r="D10" s="3">
+        <v>45653</v>
+      </c>
+      <c r="E10">
+        <v>8.8300000000000003E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="3">
+        <v>45624</v>
+      </c>
+      <c r="B11">
+        <v>0.08</v>
+      </c>
+      <c r="C11" t="s">
+        <v>75</v>
+      </c>
+      <c r="D11" s="3">
+        <v>45625</v>
+      </c>
+      <c r="E11">
+        <v>9.1399999999999995E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="3">
+        <v>45595</v>
+      </c>
+      <c r="B12">
+        <v>0.08</v>
+      </c>
+      <c r="C12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D12" s="3">
+        <v>45596</v>
+      </c>
+      <c r="E12">
+        <v>8.8200000000000001E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="3">
+        <v>45562</v>
+      </c>
+      <c r="B13">
+        <v>0.08</v>
+      </c>
+      <c r="C13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D13" s="3">
+        <v>45565</v>
+      </c>
+      <c r="E13">
+        <v>8.9899999999999994E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="3">
+        <v>45533</v>
+      </c>
+      <c r="B14">
+        <v>0.08</v>
+      </c>
+      <c r="C14" t="s">
+        <v>75</v>
+      </c>
+      <c r="D14" s="3">
+        <v>45534</v>
+      </c>
+      <c r="E14">
+        <v>9.1899999999999996E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="3">
+        <v>45503</v>
+      </c>
+      <c r="B15">
+        <v>0.08</v>
+      </c>
+      <c r="C15" t="s">
+        <v>75</v>
+      </c>
+      <c r="D15" s="3">
+        <v>45504</v>
+      </c>
+      <c r="E15">
+        <v>9.74E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="3">
+        <v>45470</v>
+      </c>
+      <c r="B16">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>75</v>
+      </c>
+      <c r="D16" s="3">
+        <v>45471</v>
+      </c>
+      <c r="E16">
+        <v>9.2200000000000004E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="3">
+        <v>45351</v>
+      </c>
+      <c r="B17">
+        <v>0.23</v>
+      </c>
+      <c r="C17" t="s">
+        <v>75</v>
+      </c>
+      <c r="D17" s="3">
+        <v>45355</v>
+      </c>
+      <c r="E17">
+        <v>7.0499999999999993E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="3">
+        <v>45349</v>
+      </c>
+      <c r="B18">
+        <v>0.08</v>
+      </c>
+      <c r="C18" t="s">
+        <v>76</v>
+      </c>
+      <c r="D18" s="3">
+        <v>45351</v>
+      </c>
+      <c r="E18">
+        <v>5.11E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="3">
+        <v>45320</v>
+      </c>
+      <c r="B19">
+        <v>0.08</v>
+      </c>
+      <c r="C19" t="s">
+        <v>76</v>
+      </c>
+      <c r="D19" s="3">
+        <v>45322</v>
+      </c>
+      <c r="E19">
+        <v>4.4200000000000003E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="3">
+        <v>45287</v>
+      </c>
+      <c r="B20">
+        <v>0.08</v>
+      </c>
+      <c r="C20" t="s">
+        <v>76</v>
+      </c>
+      <c r="D20" s="3">
+        <v>45289</v>
+      </c>
+      <c r="E20">
+        <v>3.7999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="3">
+        <v>45258</v>
+      </c>
+      <c r="B21">
+        <v>0.08</v>
+      </c>
+      <c r="C21" t="s">
+        <v>75</v>
+      </c>
+      <c r="D21" s="3">
+        <v>45260</v>
+      </c>
+      <c r="E21">
+        <v>3.4599999999999999E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="3">
+        <v>45226</v>
+      </c>
+      <c r="B22">
+        <v>0.08</v>
+      </c>
+      <c r="C22" t="s">
+        <v>76</v>
+      </c>
+      <c r="D22" s="3">
+        <v>45230</v>
+      </c>
+      <c r="E22">
+        <v>2.8899999999999999E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="3">
+        <v>45196</v>
+      </c>
+      <c r="B23">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="C23" t="s">
+        <v>76</v>
+      </c>
+      <c r="D23" s="3">
+        <v>45198</v>
+      </c>
+      <c r="E23">
+        <v>9.2700000000000005E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="3">
+        <v>45167</v>
+      </c>
+      <c r="B24">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="C24" t="s">
+        <v>76</v>
+      </c>
+      <c r="D24" s="3">
+        <v>45169</v>
+      </c>
+      <c r="E24">
+        <v>8.1299999999999997E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="3">
+        <v>45134</v>
+      </c>
+      <c r="B25">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>76</v>
+      </c>
+      <c r="D25" s="3">
+        <v>45138</v>
+      </c>
+      <c r="E25">
+        <v>8.7900000000000006E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="3">
+        <v>45014</v>
+      </c>
+      <c r="B26">
+        <v>0.09</v>
+      </c>
+      <c r="C26" t="s">
+        <v>75</v>
+      </c>
+      <c r="D26" s="3">
+        <v>45016</v>
+      </c>
+      <c r="E26">
+        <v>0.1032</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="3">
+        <v>44979</v>
+      </c>
+      <c r="B27">
+        <v>0.34</v>
+      </c>
+      <c r="C27" t="s">
+        <v>75</v>
+      </c>
+      <c r="D27" s="3">
+        <v>44981</v>
+      </c>
+      <c r="E27">
+        <v>9.4600000000000004E-2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="3">
+        <v>44953</v>
+      </c>
+      <c r="B28">
+        <v>0.09</v>
+      </c>
+      <c r="C28" t="s">
+        <v>76</v>
+      </c>
+      <c r="D28" s="3">
+        <v>44957</v>
+      </c>
+      <c r="E28">
+        <v>8.1000000000000003E-2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" s="3">
+        <v>44923</v>
+      </c>
+      <c r="B29">
+        <v>0.08</v>
+      </c>
+      <c r="C29" t="s">
+        <v>75</v>
+      </c>
+      <c r="D29" s="3">
+        <v>44925</v>
+      </c>
+      <c r="E29">
+        <v>7.8600000000000003E-2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" s="3">
+        <v>44893</v>
+      </c>
+      <c r="B30">
+        <v>0.08</v>
+      </c>
+      <c r="C30" t="s">
+        <v>75</v>
+      </c>
+      <c r="D30" s="3">
+        <v>44895</v>
+      </c>
+      <c r="E30">
+        <v>8.0600000000000005E-2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="3">
+        <v>44861</v>
+      </c>
+      <c r="B31">
+        <v>0.08</v>
+      </c>
+      <c r="C31" t="s">
+        <v>75</v>
+      </c>
+      <c r="D31" s="3">
+        <v>44865</v>
+      </c>
+      <c r="E31">
+        <v>8.0199999999999994E-2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="3">
+        <v>44812</v>
+      </c>
+      <c r="B32">
+        <v>0.08</v>
+      </c>
+      <c r="C32" t="s">
+        <v>75</v>
+      </c>
+      <c r="D32" s="3">
+        <v>44816</v>
+      </c>
+      <c r="E32">
+        <v>8.5400000000000004E-2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="3">
+        <v>44802</v>
+      </c>
+      <c r="B33">
+        <v>0.08</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33" s="3">
+        <v>44804</v>
+      </c>
+      <c r="E33">
+        <v>7.8700000000000006E-2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="3">
+        <v>44769</v>
+      </c>
+      <c r="B34">
+        <v>0.08</v>
+      </c>
+      <c r="C34" t="s">
+        <v>75</v>
+      </c>
+      <c r="D34" s="3">
+        <v>44771</v>
+      </c>
+      <c r="E34">
+        <v>7.8200000000000006E-2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="3">
+        <v>44740</v>
+      </c>
+      <c r="B35">
+        <v>0.08</v>
+      </c>
+      <c r="C35" t="s">
+        <v>75</v>
+      </c>
+      <c r="D35" s="3">
+        <v>44742</v>
+      </c>
+      <c r="E35">
+        <v>7.7100000000000002E-2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" s="3">
+        <v>44708</v>
+      </c>
+      <c r="B36">
+        <v>0.08</v>
+      </c>
+      <c r="C36" t="s">
+        <v>75</v>
+      </c>
+      <c r="D36" s="3">
+        <v>44712</v>
+      </c>
+      <c r="E36">
+        <v>6.9500000000000006E-2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" s="3">
+        <v>44678</v>
+      </c>
+      <c r="B37">
+        <v>0.08</v>
+      </c>
+      <c r="C37" t="s">
+        <v>75</v>
+      </c>
+      <c r="D37" s="3">
+        <v>44680</v>
+      </c>
+      <c r="E37">
+        <v>6.0999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" s="3">
+        <v>44629</v>
+      </c>
+      <c r="B38">
+        <v>0.08</v>
+      </c>
+      <c r="C38" t="s">
+        <v>75</v>
+      </c>
+      <c r="D38" s="3">
+        <v>44631</v>
+      </c>
+      <c r="E38">
+        <v>5.6300000000000003E-2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" s="3">
+        <v>44616</v>
+      </c>
+      <c r="B39">
+        <v>0.08</v>
+      </c>
+      <c r="C39" t="s">
+        <v>75</v>
+      </c>
+      <c r="D39" s="3">
+        <v>44620</v>
+      </c>
+      <c r="E39">
+        <v>4.8800000000000003E-2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" s="3">
+        <v>44588</v>
+      </c>
+      <c r="B40">
+        <v>0.08</v>
+      </c>
+      <c r="C40" t="s">
+        <v>75</v>
+      </c>
+      <c r="D40" s="3">
+        <v>44592</v>
+      </c>
+      <c r="E40">
+        <v>4.2099999999999999E-2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="3">
+        <v>44559</v>
+      </c>
+      <c r="B41">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="C41" t="s">
+        <v>75</v>
+      </c>
+      <c r="D41" s="3">
+        <v>44561</v>
+      </c>
+      <c r="E41">
+        <v>3.5999999999999997E-2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" s="3">
+        <v>44526</v>
+      </c>
+      <c r="B42">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>75</v>
+      </c>
+      <c r="D42" s="3">
+        <v>44530</v>
+      </c>
+      <c r="E42">
+        <v>3.0200000000000001E-2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" s="3">
+        <v>44496</v>
+      </c>
+      <c r="B43">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="C43" t="s">
+        <v>75</v>
+      </c>
+      <c r="D43" s="3">
+        <v>44498</v>
+      </c>
+      <c r="E43">
+        <v>7.6399999999999996E-2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" s="3">
+        <v>44467</v>
+      </c>
+      <c r="B44">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="C44" t="s">
+        <v>76</v>
+      </c>
+      <c r="D44" s="3">
+        <v>44469</v>
+      </c>
+      <c r="E44">
+        <v>7.7700000000000005E-2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" s="3">
+        <v>44435</v>
+      </c>
+      <c r="B45">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="C45" t="s">
+        <v>76</v>
+      </c>
+      <c r="D45" s="3">
+        <v>44439</v>
+      </c>
+      <c r="E45">
+        <v>7.9500000000000001E-2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" s="3">
+        <v>44405</v>
+      </c>
+      <c r="B46">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="C46" t="s">
+        <v>76</v>
+      </c>
+      <c r="D46" s="3">
+        <v>44407</v>
+      </c>
+      <c r="E46">
+        <v>8.1699999999999995E-2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" s="3">
+        <v>44375</v>
+      </c>
+      <c r="B47">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="C47" t="s">
+        <v>75</v>
+      </c>
+      <c r="D47" s="3">
+        <v>44377</v>
+      </c>
+      <c r="E47">
+        <v>8.0299999999999996E-2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" s="3">
+        <v>44343</v>
+      </c>
+      <c r="B48">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="C48" t="s">
+        <v>75</v>
+      </c>
+      <c r="D48" s="3">
+        <v>44347</v>
+      </c>
+      <c r="E48">
+        <v>8.6900000000000005E-2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" s="3">
+        <v>44314</v>
+      </c>
+      <c r="B49">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49" s="3">
+        <v>44316</v>
+      </c>
+      <c r="E49">
+        <v>8.8999999999999996E-2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" s="3">
+        <v>44265</v>
+      </c>
+      <c r="B50">
+        <v>0.08</v>
+      </c>
+      <c r="C50" t="s">
+        <v>75</v>
+      </c>
+      <c r="D50" s="3">
+        <v>44267</v>
+      </c>
+      <c r="E50">
+        <v>9.2100000000000001E-2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" s="3">
+        <v>44251</v>
+      </c>
+      <c r="B51">
+        <v>0.08</v>
+      </c>
+      <c r="C51" t="s">
+        <v>75</v>
+      </c>
+      <c r="D51" s="3">
+        <v>44253</v>
+      </c>
+      <c r="E51">
+        <v>8.3199999999999996E-2</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" s="3">
+        <v>44223</v>
+      </c>
+      <c r="B52">
+        <v>0.08</v>
+      </c>
+      <c r="C52" t="s">
+        <v>75</v>
+      </c>
+      <c r="D52" s="3">
+        <v>44225</v>
+      </c>
+      <c r="E52">
+        <v>9.4200000000000006E-2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" s="3">
+        <v>44194</v>
+      </c>
+      <c r="B53">
+        <v>0.09</v>
+      </c>
+      <c r="C53" t="s">
+        <v>75</v>
+      </c>
+      <c r="D53" s="3">
+        <v>44196</v>
+      </c>
+      <c r="E53">
+        <v>8.5000000000000006E-2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" s="3">
+        <v>44161</v>
+      </c>
+      <c r="B54">
+        <v>0.09</v>
+      </c>
+      <c r="C54" t="s">
+        <v>75</v>
+      </c>
+      <c r="D54" s="3">
+        <v>44165</v>
+      </c>
+      <c r="E54">
+        <v>7.6399999999999996E-2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55" s="3">
+        <v>44132</v>
+      </c>
+      <c r="B55">
+        <v>0.09</v>
+      </c>
+      <c r="C55" t="s">
+        <v>75</v>
+      </c>
+      <c r="D55" s="3">
+        <v>44134</v>
+      </c>
+      <c r="E55">
+        <v>7.8100000000000003E-2</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" s="3">
+        <v>44102</v>
+      </c>
+      <c r="B56">
+        <v>0.09</v>
+      </c>
+      <c r="C56" t="s">
+        <v>75</v>
+      </c>
+      <c r="D56" s="3">
+        <v>44104</v>
+      </c>
+      <c r="E56">
+        <v>7.22E-2</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57" s="3">
+        <v>44070</v>
+      </c>
+      <c r="B57">
+        <v>0.09</v>
+      </c>
+      <c r="C57" t="s">
+        <v>75</v>
+      </c>
+      <c r="D57" s="3">
+        <v>44074</v>
+      </c>
+      <c r="E57">
+        <v>9.3100000000000002E-2</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58" s="3">
+        <v>44041</v>
+      </c>
+      <c r="B58">
+        <v>0.09</v>
+      </c>
+      <c r="C58" t="s">
+        <v>75</v>
+      </c>
+      <c r="D58" s="3">
+        <v>44043</v>
+      </c>
+      <c r="E58">
+        <v>8.3299999999999999E-2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" s="3">
+        <v>44008</v>
+      </c>
+      <c r="B59">
+        <v>0.09</v>
+      </c>
+      <c r="C59" t="s">
+        <v>75</v>
+      </c>
+      <c r="D59" s="3">
+        <v>44012</v>
+      </c>
+      <c r="E59">
+        <v>0.104</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" s="3">
+        <v>43978</v>
+      </c>
+      <c r="B60">
+        <v>0.09</v>
+      </c>
+      <c r="C60" t="s">
+        <v>75</v>
+      </c>
+      <c r="D60" s="3">
+        <v>43980</v>
+      </c>
+      <c r="E60">
+        <v>9.1399999999999995E-2</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61" s="3">
+        <v>43949</v>
+      </c>
+      <c r="B61">
+        <v>0.09</v>
+      </c>
+      <c r="C61" t="s">
+        <v>75</v>
+      </c>
+      <c r="D61" s="3">
+        <v>43951</v>
+      </c>
+      <c r="E61">
+        <v>9.2399999999999996E-2</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" s="3">
+        <v>43882</v>
+      </c>
+      <c r="B62">
+        <v>0.17</v>
+      </c>
+      <c r="C62" t="s">
+        <v>75</v>
+      </c>
+      <c r="D62" s="3">
+        <v>43886</v>
+      </c>
+      <c r="E62">
+        <v>6.4699999999999994E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2920B5B7-5BAB-44A1-8A1D-9FB19177ABE2}">
   <dimension ref="A1:E23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6856,478 +7366,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B54206EA-71E2-4EF2-8BA5-37630DBAD1A4}">
-  <dimension ref="A1:E27"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.5703125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>82</v>
-      </c>
-      <c r="B1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C1" t="s">
-        <v>82</v>
-      </c>
-      <c r="D1" t="s">
-        <v>82</v>
-      </c>
-      <c r="E1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>72</v>
-      </c>
-      <c r="B2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D2" t="s">
-        <v>79</v>
-      </c>
-      <c r="E2" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="3">
-        <v>45834</v>
-      </c>
-      <c r="B3">
-        <v>0.61</v>
-      </c>
-      <c r="C3" t="s">
-        <v>74</v>
-      </c>
-      <c r="D3" s="3">
-        <v>45835</v>
-      </c>
-      <c r="E3">
-        <v>7.9500000000000001E-2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="3">
-        <v>45728</v>
-      </c>
-      <c r="B4">
-        <v>0.53</v>
-      </c>
-      <c r="C4" t="s">
-        <v>74</v>
-      </c>
-      <c r="D4" s="3">
-        <v>45729</v>
-      </c>
-      <c r="E4">
-        <v>6.83E-2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="3">
-        <v>45686</v>
-      </c>
-      <c r="B5">
-        <v>0.53</v>
-      </c>
-      <c r="C5" t="s">
-        <v>74</v>
-      </c>
-      <c r="D5" s="3">
-        <v>45687</v>
-      </c>
-      <c r="E5">
-        <v>6.5100000000000005E-2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="3">
-        <v>45561</v>
-      </c>
-      <c r="B6">
-        <v>0.53</v>
-      </c>
-      <c r="C6" t="s">
-        <v>74</v>
-      </c>
-      <c r="D6" s="3">
-        <v>45562</v>
-      </c>
-      <c r="E6">
-        <v>6.6100000000000006E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="3">
-        <v>45457</v>
-      </c>
-      <c r="B7">
-        <v>0.53</v>
-      </c>
-      <c r="C7" t="s">
-        <v>74</v>
-      </c>
-      <c r="D7" s="3">
-        <v>45460</v>
-      </c>
-      <c r="E7">
-        <v>6.83E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="3">
-        <v>45363</v>
-      </c>
-      <c r="B8">
-        <v>0.68</v>
-      </c>
-      <c r="C8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D8" s="3">
-        <v>45365</v>
-      </c>
-      <c r="E8">
-        <v>8.0500000000000002E-2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="3">
-        <v>45357</v>
-      </c>
-      <c r="B9">
-        <v>0.53</v>
-      </c>
-      <c r="C9" t="s">
-        <v>74</v>
-      </c>
-      <c r="D9" s="3">
-        <v>45359</v>
-      </c>
-      <c r="E9">
-        <v>6.0299999999999999E-2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="3">
-        <v>45317</v>
-      </c>
-      <c r="B10">
-        <v>0.53</v>
-      </c>
-      <c r="C10" t="s">
-        <v>74</v>
-      </c>
-      <c r="D10" s="3">
-        <v>45321</v>
-      </c>
-      <c r="E10">
-        <v>6.2600000000000003E-2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="3">
-        <v>45195</v>
-      </c>
-      <c r="B11">
-        <v>0.53</v>
-      </c>
-      <c r="C11" t="s">
-        <v>74</v>
-      </c>
-      <c r="D11" s="3">
-        <v>45197</v>
-      </c>
-      <c r="E11">
-        <v>6.8599999999999994E-2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="3">
-        <v>45091</v>
-      </c>
-      <c r="B12">
-        <v>0.53</v>
-      </c>
-      <c r="C12" t="s">
-        <v>74</v>
-      </c>
-      <c r="D12" s="3">
-        <v>45093</v>
-      </c>
-      <c r="E12">
-        <v>7.0099999999999996E-2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="3">
-        <v>44993</v>
-      </c>
-      <c r="B13">
-        <v>0.88</v>
-      </c>
-      <c r="C13" t="s">
-        <v>81</v>
-      </c>
-      <c r="D13" s="3">
-        <v>44995</v>
-      </c>
-      <c r="E13">
-        <v>9.3700000000000006E-2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="3">
-        <v>44986</v>
-      </c>
-      <c r="B14">
-        <v>0.5</v>
-      </c>
-      <c r="C14" t="s">
-        <v>74</v>
-      </c>
-      <c r="D14" s="3">
-        <v>44988</v>
-      </c>
-      <c r="E14">
-        <v>6.3700000000000007E-2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="3">
-        <v>44952</v>
-      </c>
-      <c r="B15">
-        <v>0.5</v>
-      </c>
-      <c r="C15" t="s">
-        <v>74</v>
-      </c>
-      <c r="D15" s="3">
-        <v>44956</v>
-      </c>
-      <c r="E15">
-        <v>6.4000000000000001E-2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="3">
-        <v>44830</v>
-      </c>
-      <c r="B16">
-        <v>0.5</v>
-      </c>
-      <c r="C16" t="s">
-        <v>74</v>
-      </c>
-      <c r="D16" s="3">
-        <v>44832</v>
-      </c>
-      <c r="E16">
-        <v>7.8200000000000006E-2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="3">
-        <v>44726</v>
-      </c>
-      <c r="B17">
-        <v>0.5</v>
-      </c>
-      <c r="C17" t="s">
-        <v>74</v>
-      </c>
-      <c r="D17" s="3">
-        <v>44728</v>
-      </c>
-      <c r="E17">
-        <v>8.2000000000000003E-2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="3">
-        <v>44629</v>
-      </c>
-      <c r="B18">
-        <v>0.48</v>
-      </c>
-      <c r="C18" t="s">
-        <v>74</v>
-      </c>
-      <c r="D18" s="3">
-        <v>44631</v>
-      </c>
-      <c r="E18">
-        <v>7.9600000000000004E-2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="3">
-        <v>44587</v>
-      </c>
-      <c r="B19">
-        <v>0.48</v>
-      </c>
-      <c r="C19" t="s">
-        <v>74</v>
-      </c>
-      <c r="D19" s="3">
-        <v>44589</v>
-      </c>
-      <c r="E19">
-        <v>7.9699999999999993E-2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="3">
-        <v>44462</v>
-      </c>
-      <c r="B20">
-        <v>0.48</v>
-      </c>
-      <c r="C20" t="s">
-        <v>74</v>
-      </c>
-      <c r="D20" s="3">
-        <v>44466</v>
-      </c>
-      <c r="E20">
-        <v>7.3599999999999999E-2</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="3">
-        <v>44358</v>
-      </c>
-      <c r="B21">
-        <v>0.48</v>
-      </c>
-      <c r="C21" t="s">
-        <v>74</v>
-      </c>
-      <c r="D21" s="3">
-        <v>44362</v>
-      </c>
-      <c r="E21">
-        <v>8.0600000000000005E-2</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="3">
-        <v>44265</v>
-      </c>
-      <c r="B22">
-        <v>0.48</v>
-      </c>
-      <c r="C22" t="s">
-        <v>74</v>
-      </c>
-      <c r="D22" s="3">
-        <v>44267</v>
-      </c>
-      <c r="E22">
-        <v>7.4200000000000002E-2</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="3">
-        <v>44222</v>
-      </c>
-      <c r="B23">
-        <v>0.47</v>
-      </c>
-      <c r="C23" t="s">
-        <v>75</v>
-      </c>
-      <c r="D23" s="3">
-        <v>44224</v>
-      </c>
-      <c r="E23">
-        <v>6.7599999999999993E-2</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="3">
-        <v>44097</v>
-      </c>
-      <c r="B24">
-        <v>0.48</v>
-      </c>
-      <c r="C24" t="s">
-        <v>75</v>
-      </c>
-      <c r="D24" s="3">
-        <v>44099</v>
-      </c>
-      <c r="E24">
-        <v>7.5800000000000006E-2</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="3">
-        <v>43992</v>
-      </c>
-      <c r="B25">
-        <v>0.48</v>
-      </c>
-      <c r="C25" t="s">
-        <v>75</v>
-      </c>
-      <c r="D25" s="3">
-        <v>43994</v>
-      </c>
-      <c r="E25">
-        <v>7.8299999999999995E-2</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="3">
-        <v>43899</v>
-      </c>
-      <c r="B26">
-        <v>0.45</v>
-      </c>
-      <c r="C26" t="s">
-        <v>75</v>
-      </c>
-      <c r="D26" s="3">
-        <v>43901</v>
-      </c>
-      <c r="E26">
-        <v>6.54E-2</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="3">
-        <v>43852</v>
-      </c>
-      <c r="B27">
-        <v>0.46</v>
-      </c>
-      <c r="C27" t="s">
-        <v>76</v>
-      </c>
-      <c r="D27" s="3">
-        <v>43854</v>
-      </c>
-      <c r="E27">
-        <v>6.3399999999999998E-2</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>